<commit_message>
Refresh sample dataset with NILM/smart-grid energy management search
Regenerated refs.bib, refs_abstract.bib, refs_full.bib,
refs_with_summary.bib, papers.json, papers.xlsx, and abstracts.md from
a new OpenAlex search, replacing the previous HVAC/YOLO/occupancy
detection sample set.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/refsfinder/papers.xlsx
+++ b/refsfinder/papers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,43 +471,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thermal Imagery Feature Extraction Techniques and the Effects on Machine Learning Models for Smart HVAC Efficiency in Building Energy</t>
+          <t>Deep Learning for IoT Big Data and Streaming Analytics: A Survey</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yaa Takyiwaa Acquaah; Balakrishna Gokaraju; Raymond Tesiero; Gregory H. Monty</t>
+          <t>Mehdi Mohammadi; Ala Al‐Fuqaha; Sameh Sorour; Mohsen Guizani</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Remote Sensing</t>
+          <t>IEEE Communications Surveys &amp; Tutorials</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/rs13193847</t>
+          <t>https://doi.org/10.1109/comst.2018.2844341</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>27</v>
+        <v>1483</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The control of thermostats of a heating, ventilation, and air-conditioning (HVAC) system installed in commercial and residential buildings remains a pertinent problem in building energy efficiency and thermal comfort research. The ability to determine the number of people at a particular time in an area is imperative for energy efficiency in order to condition only occupied regions and thermally deficient regions. In this study of the best features comparison for detecting the number of people i...</t>
+          <t>In the era of the Internet of Things (IoT), an enormous amount of sensing devices collect and/or generate various sensory data over time for a wide range of fields and applications. Based on the nature of the application, these devices will result in big or fast/real-time data streams. Applying analytics over such data streams to discover new information, predict future insights, and make control decisions is a crucial process that makes IoT a worthy paradigm for businesses and a quality-of-life...</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Artificial intelligence, Computer science, Pattern recognition (psychology), Wavelet, Support vector machine, Transfer of learning</t>
+          <t>Big data, Computer science, Analytics, Data science, Internet of Things, deep learning</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3204008348</t>
+          <t>https://openalex.org/W2772457693</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -519,43 +519,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A high-fidelity residential building occupancy detection dataset</t>
+          <t>Deep Learning for Edge Computing Applications: A State-of-the-Art Survey</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Margarite Jacoby; Sin Yong Tan; Gregor P. Henze; Soumik Sarkar</t>
+          <t>Fangxin Wang; Miao Zhang; Xiangxiang Wang; Xiaoqiang Ma; Jiangchuan Liu</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Scientific Data</t>
+          <t>IEEE Access</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41597-021-01055-x</t>
+          <t>https://doi.org/10.1109/access.2020.2982411</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>30</v>
+        <v>263</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>This paper describes development of a data acquisition system used to capture a range of occupancy related modalities from single-family residences, along with the dataset that was generated. The publicly available dataset includes: grayscale images at 32-by-32 pixels, captured every second; audio files, which have undergone processing to remove personally identifiable information; indoor environmental readings, captured every ten seconds; and ground truth binary occupancy status. The data acqui...</t>
+          <t>With the booming development of Internet-of-Things (IoT) and communication technologies such as 5G, our future world is envisioned as an interconnected entity where billions of devices will provide uninterrupted service to our daily lives and the industry. Meanwhile, these devices will generate massive amounts of valuable data at the network edge, calling for not only instant data processing but also intelligent data analysis in order to fully unleash the potential of the edge big data. Both the...</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Occupancy, Computer science, Ground truth, Fidelity, Modalities, Ranging</t>
+          <t>Computer science, Edge computing, Cloud computing, Edge device, Deep learning, edge computing</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3210294652</t>
+          <t>https://openalex.org/W3013557734</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -567,43 +567,43 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deep Learning-Based Industry 4.0 and Internet of Things towards Effective Energy Management for Smart Buildings</t>
+          <t>The Rise of Agentic AI: A Review of Definitions, Frameworks, Architectures, Applications, Evaluation Metrics, and Challenges</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mahmoud Elsisi; Minh‐Quang Tran; Karar Mahmoud; Matti Lehtonen; Mohamed M. F. Darwish</t>
+          <t>Ajay Bandi; Bhavani Kongari; Roshini Naguru; Sahitya Pasnoor; Sri Vidya Vilipala</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Future Internet</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s21041038</t>
+          <t>https://doi.org/10.3390/fi17090404</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Worldwide, energy consumption and saving represent the main challenges for all sectors, most importantly in industrial and domestic sectors. The internet of things (IoT) is a new technology that establishes the core of Industry 4.0. The IoT enables the sharing of signals between devices and machines via the internet. Besides, the IoT system enables the utilization of artificial intelligence (AI) techniques to manage and control the signals between different machines based on intelligence decisio...</t>
+          <t>Agentic AI systems are a recently emerged and important approach that goes beyond traditional AI, generative AI, and autonomous systems by focusing on autonomy, adaptability, and goal-driven reasoning. This study provides a clear review of agentic AI systems by bringing together their definitions, frameworks, and architectures, and by comparing them with related areas like generative AI, autonomic computing, and multi-agent systems. To do this, we reviewed 143 primary studies on current LLM-base...</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Energy consumption, Computer science, Deep learning, Dashboard, Air conditioning, Internet of Things</t>
+          <t>Computer science, Artificial intelligence, Data science, Machine learning, Software engineering, agentic AI</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3127713043</t>
+          <t>https://openalex.org/W4414023998</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -615,43 +615,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Occupancy heat gain detection and prediction using deep learning approach for reducing building energy demand</t>
+          <t>Deep Learning-Based Industry 4.0 and Internet of Things towards Effective Energy Management for Smart Buildings</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paige Wenbin Tien; Shuangyu Wei; John Kaiser Calautit; Jo Darkwa; Christopher J. Wood</t>
+          <t>Mahmoud Elsisi; Minh‐Quang Tran; Karar Mahmoud; Matti Lehtonen; Mohamed M. F. Darwish</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Journal of Sustainable Development of Energy Water and Environment Systems</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.13044/j.sdewes.d8.0378</t>
+          <t>https://doi.org/10.3390/s21041038</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>21</v>
+        <v>175</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The use of fixed or scheduled setpoints combined with varying occupancy patterns in buildings could lead to spaces being over or under-conditioned, which may lead to significant waste in energy consumption. The present study aims to develop a vision-based deep learning method for real-time occupancy activity detection and recognition. The method enables predicting and generating real-time heat gain data, which can inform building energy management systems and heating, ventilation, and air-condit...</t>
+          <t>Worldwide, energy consumption and saving represent the main challenges for all sectors, most importantly in industrial and domestic sectors. The internet of things (IoT) is a new technology that establishes the core of Industry 4.0. The IoT enables the sharing of signals between devices and machines via the internet. Besides, the IoT system enables the utilization of artificial intelligence (AI) techniques to manage and control the signals between different machines based on intelligence decisio...</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>HVAC, Occupancy, Energy consumption, Air conditioning, Deep learning, Computer science</t>
+          <t>Energy consumption, Computer science, Deep learning, Dashboard, Air conditioning, smart buildings</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3099488169</t>
+          <t>https://openalex.org/W3127713043</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Energy management, Energy (signal processing), Energy system, Architectural engineering, Environmental economics, Computer science</t>
+          <t>Energy management, Energy (signal processing), Energy system, Architectural engineering, Environmental economics, building energy management systems</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -704,46 +704,50 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Enhancing Energy Efficiency in Commercial Office Buildings: A Smart IoT and Machine Vision Approach</t>
+          <t>Application of deep learning in facility management and maintenance for heating, ventilation, and air conditioning</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sushrut Madhav Patankar; Raju Kumar Swami; Sameer Nanivadekar</t>
+          <t>Mirza Rayana Sanzana; Tomás Maul; Jing Ying Wong; Mostafa Osama Mostafa Abdulrazic; Chun-Chieh Yip</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>2022</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Automation in Construction</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/wconf61366.2024.10691999</t>
+          <t>https://doi.org/10.1016/j.autcon.2022.104445</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Commercial office buildings often waste substantial energy due to the inefficient use of HVAC and lighting systems. This paper introduces an innovative Internet of Things (IoT) and Machine Vision-based system to combat this issue and improve energy efficiency. The system combines real-time occupancy detection using the You Only Look Once (YOLO) object detection method with CCTV footage obtained through the ESP32 cam module. Additionally, machine vision technology evaluates ambient light conditio...</t>
+          <t>Despite the promising results of deep learning research, construction industry applications are still limited. Facility Management (FM) in construction has yet to take full advantage of the efficiency of deep learning techniques in daily operations and maintenance. Heating, Ventilation, and Air Conditioning (HVAC) is a major part of Facility Management and Maintenance (FMM) operations, and an occasional HVAC malfunction can lead to a huge monetary loss. The application of deep learning technique...</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Efficient energy use, Internet of Things, Computer science, Machine vision, Architectural engineering, Energy (signal processing)</t>
+          <t>HVAC, Deep learning, Air conditioning, Predictive maintenance, Computer science, deep learning</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4403126293</t>
+          <t>https://openalex.org/W4283328341</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -755,43 +759,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Data-Driven Ventilation and Energy Optimization in Smart Office Buildings: Insights from a High-Resolution Occupancy and Indoor Climate Dataset</t>
+          <t>A review of the Digital Twin technology for fault detection in buildings</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Haidar Hosamo; Silvia Mazzetto</t>
+          <t>Haidar Hosamo; Henrik Kofoed Nielsen; Ammar Alnmr; Paul Ragnar Svennevig; Kjeld Svidt</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Frontiers in Built Environment</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su17010058</t>
+          <t>https://doi.org/10.3389/fbuil.2022.1013196</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>This paper explores innovative approaches to reducing energy consumption in building ventilation systems through the implementation of adaptive control strategies. Using a publicly available high-resolution dataset spanning a full year, the study integrates real-time data on occupancy, CO2 levels, temperature, window state, and external environmental conditions. Notably, occupancy data derived from computer vision-based detection using the YOLOv5 algorithm provides an unprecedented level of gran...</t>
+          <t>This study aims to evaluate the utilization of technology known as Digital Twin for fault detection in buildings. The strategy consisted of studying existing applications, difficulties, and possibilities that come with it. The Digital Twin technology is one of the most intriguing newly discovered technologies rapidly evolving; however, some problems still need to be addressed. First, using Digital Twins to detect building faults to prevent future failures and cutting overall costs by improving b...</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Occupancy, Ventilation (architecture), Architectural engineering, Environmental science, Energy (signal processing), Computer science</t>
+          <t>Fault detection and isolation, Fault (geology), Incentive, Engineering, Computer science, digital twin</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4405781739</t>
+          <t>https://openalex.org/W4308578406</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -803,43 +807,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A Practical Multi-Sensor Cooling Demand Estimation Approach Based on Visual, Indoor and Outdoor Information Sensing</t>
+          <t>An IoT-Based Smart Building Solution for Indoor Environment Management and Occupants Prediction</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Junqi Wang; Norman C. F. Tse; Tin Yan Poon; John Yau Chung Chan</t>
+          <t>Alessandro Floris; Simone Porcu; Roberto Girau; Luigi Atzori</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Energies</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s18113591</t>
+          <t>https://doi.org/10.3390/en14102959</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The operating efficiency of heating, ventilation and air conditioning (HVAC) system is critical for building energy performance. Demand-based control is an efficient HVAC operating strategy, which can provide an appropriate level of HVAC services based on the recognition of actual cooling "demand." The cooling demand primarily relies on the accurate detection of occupancy. The current researches of demand-based HVAC control tend to detect the occupant count using cameras or other sensors, which ...</t>
+          <t>Smart buildings use Internet of Things (IoT) sensors for monitoring indoor environmental parameters, such as temperature, humidity, luminosity, and air quality. Due to the huge amount of data generated by these sensors, data analytics and machine learning techniques are needed to extract useful and interesting insights, which provide the input for the building optimization in terms of energy-saving, occupants’ health and comfort. In this paper, we propose an IoT-based smart building (SB) solutio...</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Estimation, Computer science, Real-time computing, Environmental science, Remote sensing, Engineering</t>
+          <t>Building automation, Computer science, Internet of Things, Dashboard, Indoor air quality, smart buildings</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2898388350</t>
+          <t>https://openalex.org/W3164648760</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -851,12 +855,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Occupancy Measurement in Under-Actuated Zones: YOLO-based Deep Learning Approach</t>
+          <t>Towards the application of machine learning in digital twin technology: a multi-scale review</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ade Syahputra; Yaddarabullah; Mohammad Faiz Azhary; Aedah Abd Rahman; Amna Saad</t>
+          <t>Luigi Nele; Giulio Mattera; Emily W. Yap; Mario Vozza; Silvestro Vespoli</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -864,30 +868,30 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>International Journal of Advanced Computer Science and Applications</t>
+          <t>Discover Applied Sciences</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://doi.org/10.14569/ijacsa.2024.0150277</t>
+          <t>https://doi.org/10.1007/s42452-024-06206-4</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The challenge of accurately detecting and identifying individuals within under-actuated zones presents a relevant research problem in occupant detection. This study aims to address the challenge of occupant detection in under-actuated zones through the utilization of the You Only Look Once version 8 (YOLO v8) object detection model. The research methodology involves a comprehensive evaluation of YOLO v8's performance across three distinct zones, where its precision, accuracy, and recall capabili...</t>
+          <t>This review article delves into the conceptual framework of digital twins and their diverse applications across research domains, highlighting the pivotal role of machine learning in shaping the development and integration of digital twin technology across multiple disciplines. Emphasising key features like multidisciplinarity and multi-scale aspects, the paper explores how data-driven techniques are employed for modelling, visualisation, monitoring, and optimisation within the digital twin fram...</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Computer science, Occupancy, Deep learning, Artificial intelligence, Real-time computing, Human–computer interaction</t>
+          <t>Scale (ratio), Computer science, Artificial intelligence, Machine learning, Data science, digital twin</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4392404415</t>
+          <t>https://openalex.org/W4402637216</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -899,16 +903,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Development of CNN-based visual recognition air conditioner for smart buildings</t>
+          <t>Artificial intelligence in construction asset management: a review of present status, challenges and future opportunities</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Qian Huang; Kangli Hao</t>
+          <t>Luca Rampini; Fulvio Re Cecconi</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -917,25 +921,25 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://doi.org/10.36680/j.itcon.2020.021</t>
+          <t>https://doi.org/10.36680/j.itcon.2022.043</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Demand-driven heating, ventilation, and air conditioning (HVAC) operations have become very attractive in energy-efficient smart buildings. Demand-oriented HVAC control largely relies on accurate detection of building occupancy levels and locations. So far, existing building occupancy detection methods have their disadvantages, and cannot fully meet the expected performance. To address this challenge, this paper proposes a visual recognition method based on convolutional neural networks (CNN), w...</t>
+          <t>The built environment is responsible for roughly 40% of global greenhouse emissions, making the sector a crucial factor for climate change and sustainability. Meanwhile, other sectors (like manufacturing) adopted Artificial Intelligence (AI) to solve complex, non-linear problems to reduce waste, inefficiency, and pollution. Therefore, many research efforts in the Architecture, Engineering, and Construction community have recently tried introducing AI into building asset management (AM) processes...</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>HVAC, Air conditioning, Occupancy, Building automation, Computer science, Convolutional neural network</t>
+          <t>Asset management, Context (archaeology), Computer science, Sustainability, Inefficiency, artificial intelligence</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3044090728</t>
+          <t>https://openalex.org/W4300960323</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -947,43 +951,43 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Modified Lightweight YOLO v8 Model for Fast and Precise Indoor Occupancy Detection</t>
+          <t>Human Action Recognition in Smart Living Services and Applications: Context Awareness, Data Availability, Personalization, and Privacy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hanyuan Zhang; Luyan Liu; Jingxue Bi; Hongbin Liu; Zetao Wen et al. (7 authors)</t>
+          <t>Giovanni Diraco; Gabriele Rescio; Andrea Caroppo; Andrea Manni; Alessandro Leone</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Applied Sciences</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/app16010335</t>
+          <t>https://doi.org/10.3390/s23136040</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fast and accurate indoor occupancy detection is critical for energy efficiency and emergency rescue in the fields of smart building and indoor positioning. However, existing image-based indoor occupancy detection models often neglect small human targets and suffer from large parameters, compromising detection accuracy, real-time performance, and deployment on resource-constrained devices. To address these issues, this study proposes a modified lightweight indoor occupancy detection model based o...</t>
+          <t>Smart living, an increasingly prominent concept, entails incorporating sophisticated technologies in homes and urban environments to elevate the quality of life for citizens. A critical success factor for smart living services and applications, from energy management to healthcare and transportation, is the efficacy of human action recognition (HAR). HAR, rooted in computer vision, seeks to identify human actions and activities using visual data and various sensor modalities. This paper extensiv...</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Occupancy, Computer science, Software deployment, Boosting (machine learning), Real-time computing, Feature (linguistics)</t>
+          <t>Personalization, Context (archaeology), Computer science, Smart city, Independent living, human action recognition</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://openalex.org/W7117459574</t>
+          <t>https://openalex.org/W4382599745</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -995,43 +999,43 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Review of modern demand control solutions and technologies for HVAC operation</t>
+          <t>Using Deep Learning in Real-Time for Clothing Classification with Connected Thermostats</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Anatolijs Borodiņecs; Jurģis Zemītis; Arturs Palcikovskis; Artūrs Ardavs; Egons Lavendelis</t>
+          <t>Adán Medina; Juana Isabel Méndez; Pedro Ponce; Therese E. Peffer; Alan Meier et al. (6 authors)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>E3S Web of Conferences</t>
+          <t>Energies</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1051/e3sconf/202339602020</t>
+          <t>https://doi.org/10.3390/en15051811</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>HVAC systems, which use traditional control strategies with fixed ventilation rates or with ventilation rate schedules, do not adjust according to the required IAQ and thermal comfort. As a result, building spaces are being over or under-ventilated. In this paper, the latest modern solutions for demand-controlled HVAC system operation are analyzed, based on the review of existing studies. Such modern technologies as human detection systems, computer vision, and neural network applications are lo...</t>
+          <t>Thermal comfort is associated with clothing insulation, conveying a level of satisfaction with the thermal surroundings. Besides, clothing insulation is commonly associated with indoor thermal comfort. However, clothing classification in smart homes might save energy when the end-user wears appropriate clothes to save energy and obtain thermal comfort. Furthermore, object detection and classification through Convolutional Neural Networks has increased over the last decade. There are real-time cl...</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HVAC, Occupancy, Computer science, Indoor air quality, Building automation, Architectural engineering</t>
+          <t>Clothing, Overfitting, MNIST database, Artificial intelligence, Computer science, clothing classification</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4380877501</t>
+          <t>https://openalex.org/W4214666716</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1043,91 +1047,91 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Deep Learning for Edge Computing Applications: A State-of-the-Art Survey</t>
+          <t>Measuring Indoor Occupancy through Environmental Sensors: A Systematic Review on Sensor Deployment</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fangxin Wang; Miao Zhang; Xiangxiang Wang; Xiaoqiang Ma; Jiangchuan Liu</t>
+          <t>Alma Mena-Martinez; Héctor G. Ceballos; Joanna Alvarado-Uribe</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IEEE Access</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/access.2020.2982411</t>
+          <t>https://doi.org/10.3390/s22103770</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>252</v>
+        <v>36</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>With the booming development of Internet-of-Things (IoT) and communication technologies such as 5G, our future world is envisioned as an interconnected entity where billions of devices will provide uninterrupted service to our daily lives and the industry. Meanwhile, these devices will generate massive amounts of valuable data at the network edge, calling for not only instant data processing but also intelligent data analysis in order to fully unleash the potential of the edge big data. Both the...</t>
+          <t>The COVID-19 pandemic has changed our common habits and lifestyle. Occupancy information is valued more now due to the restrictions put in place to reduce the spread of the virus. Over the years, several authors have developed methods and algorithms to detect/estimate occupancy in enclosed spaces. Similarly, different types of sensors have been installed in the places to allow this measurement. However, new researchers and practitioners often find it difficult to estimate the number of sensors t...</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Computer science, Edge computing, Cloud computing, Edge device, Deep learning, Leverage (statistics)</t>
+          <t>Occupancy, Software deployment, Computer science, Wireless sensor network, Environmental monitoring, indoor occupancy detection</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3013557734</t>
+          <t>https://openalex.org/W4280654091</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>An IoT-Based Smart Building Solution for Indoor Environment Management and Occupants Prediction</t>
+          <t>Clothing Insulation Rate and Metabolic Rate Estimation for Individual Thermal Comfort Assessment in Real Life</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alessandro Floris; Simone Porcu; Roberto Girau; Luigi Atzori</t>
+          <t>Jinsong Liu; Isak Worre Foged; Thomas Baltzer Moeslund</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Energies</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en14102959</t>
+          <t>https://doi.org/10.3390/s22020619</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Smart buildings use Internet of Things (IoT) sensors for monitoring indoor environmental parameters, such as temperature, humidity, luminosity, and air quality. Due to the huge amount of data generated by these sensors, data analytics and machine learning techniques are needed to extract useful and interesting insights, which provide the input for the building optimization in terms of energy-saving, occupants’ health and comfort. In this paper, we propose an IoT-based smart building (SB) solutio...</t>
+          <t>Satisfactory indoor thermal environments can improve working efficiencies of office staff. To build such satisfactory indoor microclimates, individual thermal comfort assessment is important, for which personal clothing insulation rate (Icl) and metabolic rate (M) need to be estimated dynamically. Therefore, this paper proposes a vision-based method. Specifically, a human tracking-by-detection framework is implemented to acquire each person’s clothing status (short-sleeved, long-sleeved), key po...</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Building automation, Computer science, Internet of Things, Dashboard, Indoor air quality, Home automation</t>
+          <t>Metabolic rate, Clothing, Thermal comfort, Estimation, Thermal manikin, metabolic rate estimation</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3164648760</t>
+          <t>https://openalex.org/W4206317890</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1139,87 +1143,91 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ODDS: Real-Time Object Detection Using Depth Sensors on Embedded GPUs</t>
+          <t>A high-fidelity residential building occupancy detection dataset</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Niluthpol Chowdhury Mithun; Sirajum Munir; Karen Guo; Charles Shelton</t>
+          <t>Margarite Jacoby; Sin Yong Tan; Gregor P. Henze; Soumik Sarkar</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2018</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>2021</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Scientific Data</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/ipsn.2018.00051</t>
+          <t>https://doi.org/10.1038/s41597-021-01055-x</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Detecting objects that are carried when someone enters or exits a room is very useful for a wide range of smart building applications including safety, security, and energy efficiency. While there has been a significant amount of work on object recognition using large-scale RGB image datasets, RGB cameras are too privacy invasive in many smart building applications and they work poorly in the dark. Additionally, deep object detection networks require powerful and expensive GPUs. We propose a nov...</t>
+          <t>This paper describes development of a data acquisition system used to capture a range of occupancy related modalities from single-family residences, along with the dataset that was generated. The publicly available dataset includes: grayscale images at 32-by-32 pixels, captured every second; audio files, which have undergone processing to remove personally identifiable information; indoor environmental readings, captured every ten seconds; and ground truth binary occupancy status. The data acqui...</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Computer science, Convolutional neural network, Object detection, RGB color model, Deep learning, Artificial intelligence</t>
+          <t>Occupancy, Computer science, Ground truth, Fidelity, Modalities, human presence detection</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2798936443</t>
+          <t>https://openalex.org/W3210294652</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>data-paper</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Privacy‐preserving labeling‐free occupancy counting sensor based on ToF camera and clustering</t>
+          <t>A Survey of FPGA-Based Vision Systems for Autonomous Cars</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jaeik Jeong; Wan‐Ki Park</t>
+          <t>David Castells‐Rufas; Vinh Ngo; Juan Borrego-Carazo; Marc Codina; Carles Sanchez et al. (7 authors)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ETRI Journal</t>
+          <t>IEEE Access</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.4218/etrij.2025-0022</t>
+          <t>https://doi.org/10.1109/access.2022.3230282</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Abstract Occupancy detection systems are crucial for optimizing energy efficiency in smart cities and buildings but often face privacy and data dependency challenges. YOLO (you only look once), a widely used real‐time detection framework, relies on identifiable image data and labeled datasets. This study proposes a privacy‐preserving, labeling‐free occupancy sensor using a time‐of‐flight (ToF) camera, and a clustering algorithm. Positioned above doorways, the ToF camera captures depth data that ...</t>
+          <t>On the road to making self-driving cars a reality, academic and industrial researchers are working hard to continue to increase safety while meeting technical and regulatory constraints Understanding the surrounding environment is a fundamental task in self-driving cars. It requires combining complex computer vision algorithms. Although state-of-the-art algorithms achieve good accuracy, their implementations often require powerful computing platforms with high power consumption. In some cases, t...</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Cluster analysis, Bounding overwatch, Computer science, Artificial intelligence, Computer vision, Energy (signal processing)</t>
+          <t>Field-programmable gate array, Computer science, Automotive industry, Implementation, Latency (audio), FPGA</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4414092520</t>
+          <t>https://openalex.org/W4312399320</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1231,12 +1239,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>An occupancy-based strategy employing computer vision for reducing cooling energy consumed in buildings</t>
+          <t>Thermal Imagery Feature Extraction Techniques and the Effects on Machine Learning Models for Smart HVAC Efficiency in Building Energy</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rania A. AlQadi; Alaa Zaghloul; Shereen A. Taie</t>
+          <t>Yaa Takyiwaa Acquaah; Balakrishna Gokaraju; Raymond Tesiero; Gregory H. Monty</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1244,30 +1252,30 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bulletin of Electrical Engineering and Informatics</t>
+          <t>Remote Sensing</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://doi.org/10.11591/eei.v10i3.3058</t>
+          <t>https://doi.org/10.3390/rs13193847</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The energy expended to cool the occupied areas by air conditioners represents a substantial share of the total energy exhausted in buildings. Therefore, developing strategies to reduce this energy is crucial. One of the preponderance strategies adopted to depreciate energy consumption in buildings is the occupancy-based strategy. In this research, an innovative model was established to achieve the goal of reducing cooling energy consumed in buildings based on occupancy-based combined with a cons...</t>
+          <t>The control of thermostats of a heating, ventilation, and air-conditioning (HVAC) system installed in commercial and residential buildings remains a pertinent problem in building energy efficiency and thermal comfort research. The ability to determine the number of people at a particular time in an area is imperative for energy efficiency in order to condition only occupied regions and thermally deficient regions. In this study of the best features comparison for detecting the number of people i...</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Setpoint, Energy consumption, Energy (signal processing), Occupancy, Air conditioning, Automotive engineering</t>
+          <t>Artificial intelligence, Computer science, Pattern recognition (psychology), Wavelet, Support vector machine, occupancy detection</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3157345320</t>
+          <t>https://openalex.org/W3204008348</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1279,43 +1287,43 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Occupant-Detection-Based Individual Control of Four-Way Air Conditioner for Sustainable Building Energy Management</t>
+          <t>Development of CNN-based visual recognition air conditioner for smart buildings</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>J H Ham; Bum‐Soo Kim; In-Woo Bae; Jaewan Joe</t>
+          <t>Qian Huang; Kangli Hao</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Journal of Information Technology in Construction</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su16177404</t>
+          <t>https://doi.org/10.36680/j.itcon.2020.021</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>In this study, individual control of a four-way air conditioner was developed based on the distribution of occupants to prevent unnecessary energy consumption during room-wide control. An occupancy detection algorithm was created in Python using YOLOv5 object recognition technology to identify the occupants’ distribution in space. Recorded video data were used to test the algorithm. A simulation case study for a building energy model was conducted, assuming that this algorithm was applied using ...</t>
+          <t>Demand-driven heating, ventilation, and air conditioning (HVAC) operations have become very attractive in energy-efficient smart buildings. Demand-oriented HVAC control largely relies on accurate detection of building occupancy levels and locations. So far, existing building occupancy detection methods have their disadvantages, and cannot fully meet the expected performance. To address this challenge, this paper proposes a visual recognition method based on convolutional neural networks (CNN), w...</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Energy consumption, Python (programming language), Thermal comfort, Air conditioning, Occupancy, Simulation</t>
+          <t>HVAC, Air conditioning, Occupancy, Building automation, Computer science, occupant detection</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4401961351</t>
+          <t>https://openalex.org/W3044090728</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1327,91 +1335,91 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Clothing Insulation Rate and Metabolic Rate Estimation for Individual Thermal Comfort Assessment in Real Life</t>
+          <t>Real operational labeled data of air handling units from office, auditorium, and hospital buildings</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jinsong Liu; Isak Worre Foged; Thomas B. Moeslund</t>
+          <t>Seunghyeon Wang</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Scientific Data</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s22020619</t>
+          <t>https://doi.org/10.1038/s41597-025-05825-9</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Satisfactory indoor thermal environments can improve working efficiencies of office staff. To build such satisfactory indoor microclimates, individual thermal comfort assessment is important, for which personal clothing insulation rate (Icl) and metabolic rate (M) need to be estimated dynamically. Therefore, this paper proposes a vision-based method. Specifically, a human tracking-by-detection framework is implemented to acquire each person’s clothing status (short-sleeved, long-sleeved), key po...</t>
+          <t>This study aims to develop comprehensive real operational datasets from three distinct building types-a large-scale office, an auditorium, and a hospital-focusing on Air Handling Units (AHUs) equipped with Constant Air Volume (CAV) systems for Automated Fault Detection and Diagnosis (AFDD). Although a consistent methodological framework was followed, data collection and preparation processes were specifically adapted to each building's unique operational characteristics. Key procedures included:...</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Metabolic rate, Clothing, Thermal comfort, Estimation, Thermal manikin, Engineering</t>
+          <t>Computer science, Identification (biology), Fault detection and isolation, Data collection, Key (lock), air handling units</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4206317890</t>
+          <t>https://openalex.org/W4413593661</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>data-paper</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Design and Validation of an Edge-AI Fire Safety System with SmartThings Integration for Accelerated Detection and Targeted Suppression</t>
+          <t>Data-Driven Ventilation and Energy Optimization in Smart Office Buildings: Insights from a High-Resolution Occupancy and Indoor Climate Dataset</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Seung-Jun Lee; Hong‐Sik Yun; Hong-Sik Yun; Sang-Hoon Lee; Sang-Hoon Lee et al. (6 authors)</t>
+          <t>Haidar Hosamo; Silvia Mazzetto</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Applied Sciences</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/app15148118</t>
+          <t>https://doi.org/10.3390/su17010058</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>This study presents the design and validation of an integrated fire safety system that leverages edge AI, hybrid sensing, and precision suppression to overcome the latency and collateral limitations of conventional smoke detection and sprinkler systems. The proposed platform features a dual-mode sensor array for early fire recognition, motorized ventilation units for rapid smoke extraction, and a 360° directional nozzle for targeted agent discharge using a residue-free clean extinguishing agent....</t>
+          <t>This paper explores innovative approaches to reducing energy consumption in building ventilation systems through the implementation of adaptive control strategies. Using a publicly available high-resolution dataset spanning a full year, the study integrates real-time data on occupancy, CO2 levels, temperature, window state, and external environmental conditions. Notably, occupancy data derived from computer vision-based detection using the YOLOv5 algorithm provides an unprecedented level of gran...</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Computer science</t>
+          <t>Occupancy, Ventilation (architecture), Architectural engineering, Environmental science, Energy (signal processing), building ventilation</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4412530877</t>
+          <t>https://openalex.org/W4405781739</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1423,43 +1431,43 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Embedded Real-Time Clothing Classifier Using One-Stage Methods for Saving Energy in Thermostats</t>
+          <t>A Practical Multi-Sensor Cooling Demand Estimation Approach Based on Visual, Indoor and Outdoor Information Sensing</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Adán Medina; Juana Isabel Méndez; Pedro Ponce; Therese Peffer; Arturo Molina</t>
+          <t>Junqi Wang; Norman C. F. Tse; Tin Yan Poon; John Yau Chung Chan</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Energies</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en15176117</t>
+          <t>https://doi.org/10.3390/s18113591</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Energy-saving is a mandatory research topic since the growing population demands additional energy yearly. Moreover, climate change requires more attention to reduce the impact of generating more CO2. As a result, some new research areas need to be explored to create innovative energy-saving alternatives in electrical devices that have high energy consumption. One research area of interest is the computer visual classification for reducing energy consumption and keeping thermal comfort in thermo...</t>
+          <t>The operating efficiency of heating, ventilation and air conditioning (HVAC) system is critical for building energy performance. Demand-based control is an efficient HVAC operating strategy, which can provide an appropriate level of HVAC services based on the recognition of actual cooling "demand." The cooling demand primarily relies on the accurate detection of occupancy. The current researches of demand-based HVAC control tend to detect the occupant count using cameras or other sensors, which ...</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Thermostat, Energy consumption, Computer science, Clothing, HVAC, Efficient energy use</t>
+          <t>Estimation, Computer science, Real-time computing, Environmental science, Remote sensing, multi-sensor fusion</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4293030513</t>
+          <t>https://openalex.org/W2898388350</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1471,43 +1479,43 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IoB Internet of Things (IoT) for Smart Built Environment (SBE): Understanding the Complexity and Contributing to Energy Efficiency; A Case Study in Mediterranean Climates</t>
+          <t>Occupancy heat gain detection and prediction using deep learning approach for reducing building energy demand</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ignacio Martínez Ruiz; Enrique Cano-Suñén; Álvaro Marco; Ángel Fernández</t>
+          <t>Paige Wenbin Tien; Shuangyu Wei; John Kaiser Calautit; Jo Darkwa; Christopher J. Wood</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Applied Sciences</t>
+          <t>Journal of Sustainable Development of Energy Water and Environment Systems</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/app15041724</t>
+          <t>https://doi.org/10.13044/j.sdewes.d8.0378</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>To meet the 2050 targets about climate change and decarbonization, accomplishing thermal comfort, Internet of Things (IoT) ecosystems are key enabling technologies to move the Built Environment (BE) towards Smart Built Environment (SBE). The first contributions of this paper conceptualise SBE from its dynamic and adaptative perspectives, considering the human habitat, and enunciate SBE as a multidimensional approach through six ways of inhabiting: defensive, projective, scientific, thermodynamic...</t>
+          <t>The use of fixed or scheduled setpoints combined with varying occupancy patterns in buildings could lead to spaces being over or under-conditioned, which may lead to significant waste in energy consumption.The present study aims to develop a vision-based deep learning method for real-time occupancy activity detection and recognition.The method enables predicting and generating real-time heat gain data, which can inform building energy management systems and heating, ventilation, and air-conditio...</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Internet of Things, Computer science, Computer security</t>
+          <t>HVAC, Occupancy, Energy consumption, Air conditioning, Deep learning, occupancy detection</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4407339412</t>
+          <t>https://openalex.org/W3099488169</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1519,91 +1527,91 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Artificial intelligence in construction asset management: a review of present status, challenges and future opportunities</t>
+          <t>An Ultra-low-power Embedded AI Fire Detection and Crowd Counting System for Indoor Areas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Luca Rampini; Fulvio Re Cecconi</t>
+          <t>Alexios Papaioannou; Charalampos S. Kouzinopoulos; Dimosthenis Ioannidis; Dimitrios K. Tzovaras</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Journal of Information Technology in Construction</t>
+          <t>ACM Transactions on Embedded Computing Systems</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://doi.org/10.36680/j.itcon.2022.043</t>
+          <t>https://doi.org/10.1145/3582433</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>The built environment is responsible for roughly 40% of global greenhouse emissions, making the sector a crucial factor for climate change and sustainability. Meanwhile, other sectors (like manufacturing) adopted Artificial Intelligence (AI) to solve complex, non-linear problems to reduce waste, inefficiency, and pollution. Therefore, many research efforts in the Architecture, Engineering, and Construction community have recently tried introducing AI into building asset management (AM) processes...</t>
+          <t>Fire incidents in residential and industrial areas are often the cause of human casualties and property damage. Although there are existing systems that detect fire and monitor the presence of people in indoor areas, research on their implementation in embedded platforms is limited. This article introduces an ultra-low-power embedded system for fire detection and crowd counting using efficient deep learning methods. For the prediction of fire occurrences, environmental and gas sensor along with ...</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Asset management, Context (archaeology), Computer science, Sustainability, Inefficiency, Asset (computer security)</t>
+          <t>Computer science, Fire detection, Deep learning, Real-time computing, Inference, fire detection</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4300960323</t>
+          <t>https://openalex.org/W4320498313</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Real operational labeled data of air handling units from office, auditorium, and hospital buildings</t>
+          <t>A ventilation early warning system (VEWS) for diaphanous workspaces considering COVID-19 and future pandemics scenarios</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Seunghyeon Wang</t>
+          <t>Gonçal Costa; Oriol Arroyo; Pablo Rueda; Alan Briones</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Scientific Data</t>
+          <t>Heliyon</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41597-025-05825-9</t>
+          <t>https://doi.org/10.1016/j.heliyon.2023.e14640</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>This study aims to develop comprehensive real operational datasets from three distinct building types-a large-scale office, an auditorium, and a hospital-focusing on Air Handling Units (AHUs) equipped with Constant Air Volume (CAV) systems for Automated Fault Detection and Diagnosis (AFDD). Although a consistent methodological framework was followed, data collection and preparation processes were specifically adapted to each building's unique operational characteristics. Key procedures included:...</t>
+          <t>The COVID-19 pandemic has generated new needs due to the associated health risks and, more specifically, its rapid infection rate. Prevention measures to avoid contagions in indoor spaces, especially in office and public buildings (e.g., hospitals, public administration, educational centres, etc.), have led to the need for adequate ventilation to dilute the possible concentration of the virus. This article presents our contribution to this new challenge, namely the Ventilation Early Warning Syst...</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Computer science, Identification (biology), Fault detection and isolation, Data collection, Key (lock), Raw data</t>
+          <t>HVAC, Workspace, Warning system, Sustainability, Architectural engineering, HVAC control</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4413593661</t>
+          <t>https://openalex.org/W4327702769</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1615,60 +1623,56 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>A Lightweight Electronic Water Pump Shell Defect Detection Method Based on Improved YOLOv5s</t>
+          <t>ODDS: Real-Time Object Detection Using Depth Sensors on Embedded GPUs</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Qunbiao Wu; Zhen Wang; Haifeng Fang; Junji Chen; Xinfeng Wan</t>
+          <t>Niluthpol Chowdhury Mithun; Sirajum Munir; Karen Guo; Charles Shelton</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Computer Systems Science and Engineering</t>
-        </is>
-      </c>
+        <v>2018</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://doi.org/10.32604/csse.2023.036239</t>
+          <t>https://doi.org/10.1109/ipsn.2018.00051</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>For surface defects in electronic water pump shells, the manual detection efficiency is low, prone to misdetection and leak detection, and encounters problems, such as uncertainty. To improve the speed and accuracy of surface defect detection, a lightweight detection method based on an improved YOLOv5s method is proposed to replace the traditional manual detection methods. In this method, the MobileNetV3 module replaces the backbone network of YOLOv5s, depth-separable convolution is introduced, ...</t>
+          <t>Detecting objects that are carried when someone enters or exits a room is very useful for a wide range of smart building applications including safety, security, and energy efficiency. While there has been a significant amount of work on object recognition using large-scale RGB image datasets, RGB cameras are too privacy invasive in many smart building applications and they work poorly in the dark. Additionally, deep object detection networks require powerful and expensive GPUs. We propose a nov...</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Computer science, Artificial intelligence, Pattern recognition (psychology)</t>
+          <t>Computer science, Convolutional neural network, Object detection, RGB color model, Deep learning, object detection</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4317906189</t>
+          <t>https://openalex.org/W2798936443</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>conference-paper</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Testing and Evaluation of Low-Cost Sensors for Developing Open Smart Campus Systems Based on IoT</t>
+          <t>Advanced Power Converters and Learning in Diverse Robotic Innovation: A Review</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pascal Neis; Dominik Warch; Max Hoppe</t>
+          <t>Rupam Singh; Varaha Satya Bharath Kurukuru; Mohammed Ali Khan</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1676,30 +1680,30 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Energies</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s23208652</t>
+          <t>https://doi.org/10.3390/en16207156</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Urbanization has led to the need for the intelligent management of various urban challenges, from traffic to energy. In this context, smart campuses and buildings emerge as microcosms of smart cities, offering both opportunities and challenges in technology and communication integration. This study sets itself apart by prioritizing sustainable, adaptable, and reusable solutions through an open-source framework and open data protocols. We utilized the Internet of Things (IoT) and cost-effective s...</t>
+          <t>This paper provides a comprehensive review of the integration of advanced power management systems and learning techniques in the field of robotics. It identifies the critical roles these areas play in reshaping the capabilities of robotic systems across diverse applications. To begin, it highlights the significance of efficient power usage in modern robotics. The paper explains how advanced power converters effectively control voltage, manage current and shape waveforms, thereby optimizing ener...</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Smart city, Computer science, Context (archaeology), Visitor pattern, Building automation, USable</t>
+          <t>Artificial intelligence, Robotics, Computer science, Flexibility (engineering), Robot, power converters</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4387874460</t>
+          <t>https://openalex.org/W4387780723</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1711,43 +1715,43 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A Survey of FPGA-Based Vision Systems for Autonomous Cars</t>
+          <t>A Review of the Potential of Drone-Based Approaches for Integrated Building Envelope Assessment</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>David Castells‐Rufas; Vinh Ngo; Juan Borrego-Carazo; Marc Codina; Carles Sanchez et al. (7 authors)</t>
+          <t>Shayan Mirzabeigi; Ryan Razkenari; Paul L. Crovella</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>IEEE Access</t>
+          <t>Buildings</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/access.2022.3230282</t>
+          <t>https://doi.org/10.3390/buildings15132230</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>On the road to making self-driving cars a reality, academic and industrial researchers are working hard to continue to increase safety while meeting technical and regulatory constraints Understanding the surrounding environment is a fundamental task in self-driving cars. It requires combining complex computer vision algorithms. Although state-of-the-art algorithms achieve good accuracy, their implementations often require powerful computing platforms with high power consumption. In some cases, t...</t>
+          <t>The urgent need for affordable and scalable building retrofit solutions has intensified due to stringent clean energy targets. Traditional building energy audits, which are essential in assessing energy performance, are often time-consuming and costly because of the extensive field analysis required. There has been a gradual shift towards the public use of drones, which present opportunities for effective remote procedures that could disrupt a variety of built environment disciplines. Drone-base...</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Field-programmable gate array, Computer science, Automotive industry, Implementation, Latency (audio), Advanced driver assistance systems</t>
+          <t>Drone, Building envelope, Envelope (radar), Systems engineering, Engineering, building energy audit</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4312399320</t>
+          <t>https://openalex.org/W4411651052</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1759,43 +1763,43 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>A Cost-Effective System for Indoor Three-Dimensional Occupant Positioning and Trajectory Reconstruction</t>
+          <t>Design and Validation of an Edge-AI Fire Safety System with SmartThings Integration for Accelerated Detection and Targeted Suppression</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Xiaomei Zhao; Shuo Li; Zhan Zhao; Honggang Li</t>
+          <t>Seung-Jun Lee; Seung-Jun Lee; Hong-Sik Yun; Yang-Bae Sim; Sang-Hoon Lee et al. (6 authors)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>Applied Sciences</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings13112832</t>
+          <t>https://doi.org/10.3390/app15148118</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Accurate indoor occupancy information extraction plays a crucial role in building energy conservation. Vision-based methods are popularly used for occupancy information extraction because of their high accuracy. However, previous vision-based methods either only provide 2D occupancy information or require expensive equipment. In this paper, we propose a cost-effective indoor occupancy information extraction system that estimates occupant positions and trajectories in 3D using a single RGB camera...</t>
+          <t>This study presents the design and validation of an integrated fire safety system that leverages edge AI, hybrid sensing, and precision suppression to overcome the latency and collateral limitations of conventional smoke detection and sprinkler systems. The proposed platform features a dual-mode sensor array for early fire recognition, motorized ventilation units for rapid smoke extraction, and a 360° directional nozzle for targeted agent discharge using a residue-free clean extinguishing agent....</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Occupancy, Computer vision, Computer science, Tracking (education), Artificial intelligence, Trajectory</t>
+          <t>Computer science, edge AI, fire safety systems, fire detection, smoke detection, probabilistic risk assessment</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4388637068</t>
+          <t>https://openalex.org/W4412530877</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1807,43 +1811,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>A novel lightweight skeletal temporal model for real-time, computationally efficient recognition of occupant thermal adaptation behavior</t>
+          <t>Embedded Real-Time Clothing Classifier Using One-Stage Methods for Saving Energy in Thermostats</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Zhe Wang; Hao Sun; John Kaiser Calautit; Mingda Yang; Jianbin Chen et al. (7 authors)</t>
+          <t>Adán Medina; Juana Isabel Méndez; Pedro Ponce; Therese E. Peffer; Arturo Molina</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Building Simulation</t>
+          <t>Energies</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12273-025-1335-6</t>
+          <t>https://doi.org/10.3390/en15176117</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Abstract Optimizing building energy systems based on real-time occupant behavior and feedback can lead to improved energy efficiency and enhanced thermal comfort in buildings. Traditional thermal comfort surveys do not provide real-time insights, while conventional sensors, such as thermal sensors, are limited in their ability to capture continuous, detailed occupancy data. Meanwhile, deep learning and computer vision have emerged as promising approaches for real-time occupancy behavior detectio...</t>
+          <t>Energy-saving is a mandatory research topic since the growing population demands additional energy yearly. Moreover, climate change requires more attention to reduce the impact of generating more CO2. As a result, some new research areas need to be explored to create innovative energy-saving alternatives in electrical devices that have high energy consumption. One research area of interest is the computer visual classification for reducing energy consumption and keeping thermal comfort in thermo...</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Adaptation (eye), Thermal, Computer science, Artificial intelligence, Engineering, Real-time computing</t>
+          <t>Thermostat, Energy consumption, Computer science, Clothing, HVAC, clothing classification</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4413874967</t>
+          <t>https://openalex.org/W4293030513</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1855,12 +1859,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>A ventilation early warning system (VEWS) for diaphanous workspaces considering COVID-19 and future pandemics scenarios</t>
+          <t>Testing and Evaluation of Low-Cost Sensors for Developing Open Smart Campus Systems Based on IoT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gonçal Costa; Oriol Arroyo; Pablo Rueda; Alan Briones</t>
+          <t>Pascal Neis; Dominik Warch; Max Hoppe</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1868,30 +1872,30 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Heliyon</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.heliyon.2023.e14640</t>
+          <t>https://doi.org/10.3390/s23208652</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>The COVID-19 pandemic has generated new needs due to the associated health risks and, more specifically, its rapid infection rate. Prevention measures to avoid contagions in indoor spaces, especially in office and public buildings (e.g., hospitals, public administration, educational centres, etc.), have led to the need for adequate ventilation to dilute the possible concentration of the virus. This article presents our contribution to this new challenge, namely the Ventilation Early Warning Syst...</t>
+          <t>Urbanization has led to the need for the intelligent management of various urban challenges, from traffic to energy. In this context, smart campuses and buildings emerge as microcosms of smart cities, offering both opportunities and challenges in technology and communication integration. This study sets itself apart by prioritizing sustainable, adaptable, and reusable solutions through an open-source framework and open data protocols. We utilized the Internet of Things (IoT) and cost-effective s...</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>HVAC, Workspace, Warning system, Sustainability, Architectural engineering, Computer science</t>
+          <t>Smart city, Computer science, Context (archaeology), Visitor pattern, Building automation, low-cost sensors</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4327702769</t>
+          <t>https://openalex.org/W4387874460</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1903,91 +1907,91 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Advanced Power Converters and Learning in Diverse Robotic Innovation: A Review</t>
+          <t>VR digital twin of office space with computer vision-based estimation of room occupancy and power consumption</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rupam Singh; Varaha Satya Bharath Kurukuru; Mohammed Ali Khan</t>
+          <t>Abhishek Mukhopadhyay; Naveen R. Talwar; Himanshu Viswakarma; G. S. Rajshekar Reddy; Shakti Srivastava et al. (7 authors)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Energies</t>
+          <t>Discover Analytics</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en16207156</t>
+          <t>https://doi.org/10.1007/s44257-024-00008-z</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>This paper provides a comprehensive review of the integration of advanced power management systems and learning techniques in the field of robotics. It identifies the critical roles these areas play in reshaping the capabilities of robotic systems across diverse applications. To begin, it highlights the significance of efficient power usage in modern robotics. The paper explains how advanced power converters effectively control voltage, manage current and shape waveforms, thereby optimizing ener...</t>
+          <t>Abstract In the past years, energy consumption has increased rapidly due to many factors, including the rise in technology adoption. This has many downfalls, from higher costs to CO $$_2$$ 2 emissions. Human activities in offices and houses represent a considerable amount of energy usage. A digital twin (DT) of an open-plan common space is created, serving the purpose of remote room occupancy monitoring and automatic detection of energy consumption. A virtual reality (VR) model is developed and ...</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Artificial intelligence, Robotics, Computer science, Flexibility (engineering), Robot, Reinforcement learning</t>
+          <t>Algorithm, Computer science, Artificial intelligence, Machine learning, Database, digital twin</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4387780723</t>
+          <t>https://openalex.org/W4394822553</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>A pilot study of occupant centric control stratum ventilation based on computer vision</t>
+          <t>A novel lightweight skeletal temporal model for real-time, computationally efficient recognition of occupant thermal adaptation behavior</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yihang Liu; Bin Yang; Zhang Lin</t>
+          <t>Zhe Wang; Hao Sun; John Kaiser Calautit; Mingda Yang; Jianbin Chen et al. (7 authors)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>E3S Web of Conferences</t>
+          <t>Building Simulation</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1051/e3sconf/202235601029</t>
+          <t>https://doi.org/10.1007/s12273-025-1335-6</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Indoor occupant information has an obvious influence on operating parameters of heating ventilation and air conditioning (HVAC) system, which further affects occupants’ thermal comfort and energy consumption. This pilot study proposes an occupant centric control (OCC) strategy for stratum ventilation (SV) to achieve demand control ventilation (DCV). Firstly, the computer vision sensing system and deep learning algorithm are used to detect the number of occupants in real time, and the accuracy of...</t>
+          <t>Abstract Optimizing building energy systems based on real-time occupant behavior and feedback can lead to improved energy efficiency and enhanced thermal comfort in buildings. Traditional thermal comfort surveys do not provide real-time insights, while conventional sensors, such as thermal sensors, are limited in their ability to capture continuous, detailed occupancy data. Meanwhile, deep learning and computer vision have emerged as promising approaches for real-time occupancy behavior detectio...</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>HVAC, Ventilation (architecture), Thermal comfort, Cooling load, Energy consumption, Automotive engineering</t>
+          <t>Adaptation (eye), Thermal, Computer science, Artificial intelligence, Engineering, thermal comfort</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4293719888</t>
+          <t>https://openalex.org/W4413874967</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1999,60 +2003,56 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Towards the application of machine learning in digital twin technology: a multi-scale review</t>
+          <t>Enhancing Energy Efficiency in Commercial Office Buildings: A Smart IoT and Machine Vision Approach</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Luigi Nele; Giulio Mattera; Emily W. Yap; Mario Vozza; Silvestro Vespoli</t>
+          <t>Sushrut Madhav Patankar; Raju Kumar Swami; Sameer Suresh Nanivadekar</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>2024</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Discover Applied Sciences</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s42452-024-06206-4</t>
+          <t>https://doi.org/10.1109/wconf61366.2024.10691999</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>This review article delves into the conceptual framework of digital twins and their diverse applications across research domains, highlighting the pivotal role of machine learning in shaping the development and integration of digital twin technology across multiple disciplines. Emphasising key features like multidisciplinarity and multi-scale aspects, the paper explores how data-driven techniques are employed for modelling, visualisation, monitoring, and optimisation within the digital twin fram...</t>
+          <t>Commercial office buildings often waste substantial energy due to the inefficient use of HVAC and lighting systems. This paper introduces an innovative Internet of Things (IoT) and Machine Vision-based system to combat this issue and improve energy efficiency. The system combines real-time occupancy detection using the You Only Look Once (YOLO) object detection method with CCTV footage obtained through the ESP32 cam module. Additionally, machine vision technology evaluates ambient light conditio...</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Scale (ratio), Computer science, Artificial intelligence, Machine learning, Data science, Human–computer interaction</t>
+          <t>Efficient energy use, Internet of Things, Computer science, Machine vision, Architectural engineering, commercial office buildings</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4402637216</t>
+          <t>https://openalex.org/W4403126293</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>conference-paper</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Human Action Recognition in Smart Living Services and Applications: Context Awareness, Data Availability, Personalization, and Privacy</t>
+          <t>Review of modern demand control solutions and technologies for HVAC operation</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Giovanni Diraco; Gabriele Rescio; Andrea Caroppo; Andrea Manni; Alessandro Leone</t>
+          <t>Anatolijs Borodiņecs; Jurģis Zemītis; Arturs Palcikovskis; Artūrs Ardavs; Egons Lavendelis</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2060,99 +2060,99 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>E3S Web of Conferences</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s23136040</t>
+          <t>https://doi.org/10.1051/e3sconf/202339602020</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Smart living, an increasingly prominent concept, entails incorporating sophisticated technologies in homes and urban environments to elevate the quality of life for citizens. A critical success factor for smart living services and applications, from energy management to healthcare and transportation, is the efficacy of human action recognition (HAR). HAR, rooted in computer vision, seeks to identify human actions and activities using visual data and various sensor modalities. This paper extensiv...</t>
+          <t>HVAC systems, which use traditional control strategies with fixed ventilation rates or with ventilation rate schedules, do not adjust according to the required IAQ and thermal comfort. As a result, building spaces are being over or under-ventilated. In this paper, the latest modern solutions for demand-controlled HVAC system operation are analyzed, based on the review of existing studies. Such modern technologies as human detection systems, computer vision, and neural network applications are lo...</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Personalization, Context (archaeology), Computer science, Smart city, Independent living, Data science</t>
+          <t>HVAC, Occupancy, Computer science, Indoor air quality, Building automation, demand-controlled ventilation</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4382599745</t>
+          <t>https://openalex.org/W4380877501</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>conference-paper</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Deep Learning for IoT Big Data and Streaming Analytics: A Survey</t>
+          <t>IoB Internet of Things (IoT) for Smart Built Environment (SBE): Understanding the Complexity and Contributing to Energy Efficiency; A Case Study in Mediterranean Climates</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mehdi Mohammadi; Ala Al‐Fuqaha; Sameh Sorour; Mohsen Guizani</t>
+          <t>Ignacio Martínez Ruiz; Enrique Cano-Suñén; Álvaro Marco; Ángel Fernández</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2018</v>
+        <v>2025</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IEEE Communications Surveys &amp; Tutorials</t>
+          <t>Applied Sciences</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/comst.2018.2844341</t>
+          <t>https://doi.org/10.3390/app15041724</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>88</v>
+        <v>4</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>In the era of the Internet of Things (IoT), an enormous amount of sensing devices collect and/or generate various sensory data over time for a wide range of fields and applications. Based on the nature of the application, these devices will result in big or fast/real-time data streams. Applying analytics over such data streams to discover new information, predict future insights, and make control decisions is a crucial process that makes IoT a worthy paradigm for businesses and a quality-of-life...</t>
+          <t>To meet the 2050 targets about climate change and decarbonization, accomplishing thermal comfort, Internet of Things (IoT) ecosystems are key enabling technologies to move the Built Environment (BE) towards Smart Built Environment (SBE). The first contributions of this paper conceptualise SBE from its dynamic and adaptative perspectives, considering the human habitat, and enunciate SBE as a multidimensional approach through six ways of inhabiting: defensive, projective, scientific, thermodynamic...</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Big data, Computer science, Analytics, Data science, Internet of Things, Data analysis</t>
+          <t>Internet of Things, Computer science, Computer security, smart built environment, energy efficiency, public buildings</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2772457693</t>
+          <t>https://openalex.org/W4407339412</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Scan-to-EDTs: Automated Generation of Energy Digital Twins from 3D Point Clouds</t>
+          <t>A Cost-Effective System for Indoor Three-Dimensional Occupant Positioning and Trajectory Reconstruction</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>O. V. Roman; Maarten Bassier; Giorgio Agugiaro; Ken Arroyo Ohori; Elisa Mariarosaria Farella et al. (6 authors)</t>
+          <t>Xiaomei Zhao; Shuo Li; Zhan Zhao; Honggang Li</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2161,25 +2161,25 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings15224060</t>
+          <t>https://doi.org/10.3390/buildings13112832</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Digital Twins (DTs) are transforming construction and energy management sectors by integrating 3D surveying, monitoring, Building Performance Simulation (BPS), and Building Energy Simulation (BES) from the earliest design or retrofit stages. Moreover, dynamic thermal simulations further support energy performance assessments by modeling indoor conditions to meet comfort and efficiency targets. However, their reliability depends on accurate, standards-compliant 3D building models, which are costl...</t>
+          <t>Accurate indoor occupancy information extraction plays a crucial role in building energy conservation. Vision-based methods are popularly used for occupancy information extraction because of their high accuracy. However, previous vision-based methods either only provide 2D occupancy information or require expensive equipment. In this paper, we propose a cost-effective indoor occupancy information extraction system that estimates occupant positions and trajectories in 3D using a single RGB camera...</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Reliability (semiconductor), Energy (signal processing), Computer science, Point cloud, Efficient energy use, Point (geometry)</t>
+          <t>Occupancy, Computer vision, Computer science, Tracking (education), Artificial intelligence, indoor occupancy detection</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4416196109</t>
+          <t>https://openalex.org/W4388637068</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2191,60 +2191,60 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Privacy-Preserving Person Detection Using Low-Resolution Infrared Cameras</t>
+          <t>Improved human image density detection with comparison of YOLOv8 depth level architecture and drop-out implementation</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Thomas Dubail; Fidel A. Guerrero Peña; Heitor R. Medeiros; Masih Aminbeidokhti; Éric Granger et al. (6 authors)</t>
+          <t>Winda Yulita; Uri Arta Ramadhani; Zunanik Mufidah; Gde KM Atmajaya; Radhinka Bagaskara et al. (7 authors)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>arXiv (Cornell University)</t>
+          <t>Journal of Soft Computing Exploration</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://doi.org/10.48550/arxiv.2209.11335</t>
+          <t>https://doi.org/10.52465/joscex.v6i1.556</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>In intelligent building management, knowing the number of people and their location in a room are important for better control of its illumination, ventilation, and heating with reduced costs and improved comfort. This is typically achieved by detecting people using compact embedded devices that are installed on the room's ceiling, and that integrate low-resolution infrared camera, which conceals each person's identity. However, for accurate detection, state-of-the-art deep learning models still...</t>
+          <t>Energy inefficiency due to Air Conditioners (AC) running in empty rooms contribute to unnecessary energy consumption and increased CO₂ emissions. This study explores how different depth levels of the YOLOv8 architecture and dropout regularization can enhance human density detection for smarter AC control systems. By evaluating model accuracy through Mean Average Precision (mAP50-95), we provide quantitative insights into how these modifications improve detection performance. Our dataset consists...</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Computer science, Artificial intelligence, Computer vision, Detector, Minimum bounding box, Computation</t>
+          <t>Architecture, Image (mathematics), Drop (telecommunication), Computer science, Artificial intelligence, YOLOv8</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4297162628</t>
+          <t>https://openalex.org/W4409512193</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Building Ventilation Optimization Through Occupant-Centered Computer Vision Analysis</t>
+          <t>A Lightweight Electronic Water Pump Shell Defect Detection Method Based on Improved YOLOv5s</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jevgēnijs Teličko; Kirill I. Bolotin</t>
+          <t>Qunbiao Wu; Zhen Wang; Haifeng Fang; Junji Chen; Xinfeng Wan</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2252,12 +2252,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Latvian Journal of Physics and Technical Sciences</t>
+          <t>Computer Systems Science and Engineering</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://doi.org/10.2478/lpts-2023-0045</t>
+          <t>https://doi.org/10.32604/csse.2023.036239</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2265,17 +2265,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Abstract Buildings consume about 40 % of all energy. Ventilation plays a significant role in both the energy consumption of buildings and the comfort of occupants. To achieve energy efficiency and comfort, smarter ventilation control algorithms can be employed, such as those with feedback based on CO 2 levels. Furthermore, by knowing the current number of people in a space, ventilation can theoretically be adjusted to maintain a constant CO 2 level without wasting energy when people are not pres...</t>
+          <t>For surface defects in electronic water pump shells, the manual detection efficiency is low, prone to misdetection and leak detection, and encounters problems, such as uncertainty. To improve the speed and accuracy of surface defect detection, a lightweight detection method based on an improved YOLOv5s method is proposed to replace the traditional manual detection methods. In this method, the MobileNetV3 module replaces the backbone network of YOLOv5s, depth-separable convolution is introduced, ...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Ventilation (architecture), Simulation, Computer science, Energy consumption, Architectural engineering, Efficient energy use</t>
+          <t>Computer science, Artificial intelligence, Pattern recognition (psychology), surface defect detection, lightweight object detection, YOLOv5</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4389505029</t>
+          <t>https://openalex.org/W4317906189</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2287,43 +2287,43 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Real-time Occupancy Detection and Tracking for HVAC Control in an Office Building</t>
+          <t>Occupancy Measurement in Under-Actuated Zones: YOLO-based Deep Learning Approach</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jun-Sub Kim; Sun Ho Kim; Moon Hyeun Jun</t>
+          <t>Ade Syahputra; Yaddarabullah Yaddarabullah; Mohammad Faiz Azhary; Aedah Binti Abd Rahman; Amna Binti Saad</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Building Simulation Conference proceedings</t>
+          <t>International Journal of Advanced Computer Science and Applications</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://doi.org/10.26868/25222708.2025.1472</t>
+          <t>https://doi.org/10.14569/ijacsa.2024.0150277</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>The efficient management of energy in office buildings is contingent upon the accurate real-time detection of occupancy. Conventional HVAC systems, often reliant on fixed schedules, struggle with inefficiency due to a mismatch with actual occupancy. While vision-based systems offer a promising solution, relying on detection-only models is insufficient, as they fail to provide reliable counts due to significant tracking errors like ID fragmentation. To address this specific limitation, this study...</t>
+          <t>The challenge of accurately detecting and identifying individuals within under-actuated zones presents a relevant research problem in occupant detection. This study aims to address the challenge of occupant detection in under-actuated zones through the utilization of the You Only Look Once version 8 (YOLO v8) object detection model. The research methodology involves a comprehensive evaluation of YOLO v8's performance across three distinct zones, where its precision, accuracy, and recall capabili...</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>HVAC, Computer science, Schedule, Inefficiency, Key (lock), Tracking (education)</t>
+          <t>Computer science, Occupancy, Deep learning, Artificial intelligence, Real-time computing, occupant detection</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4416704736</t>
+          <t>https://openalex.org/W4392404415</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2335,12 +2335,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>A Review of the Potential of Drone-Based Approaches for Integrated Building Envelope Assessment</t>
+          <t>Privacy‐preserving labeling‐free occupancy counting sensor based on ToF camera and clustering</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Shayan Mirzabeigi; Ryan Razkenari; Paul Crovella</t>
+          <t>Jaeik Jeong; Wan–Ki Park</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2348,173 +2348,317 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>ETRI Journal</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings15132230</t>
+          <t>https://doi.org/10.4218/etrij.2025-0022</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>The urgent need for affordable and scalable building retrofit solutions has intensified due to stringent clean energy targets. Traditional building energy audits, which are essential in assessing energy performance, are often time-consuming and costly because of the extensive field analysis required. There has been a gradual shift towards the public use of drones, which present opportunities for effective remote procedures that could disrupt a variety of built environment disciplines. Drone-base...</t>
+          <t>Abstract Occupancy detection systems are crucial for optimizing energy efficiency in smart cities and buildings but often face privacy and data dependency challenges. YOLO (you only look once), a widely used real‐time detection framework, relies on identifiable image data and labeled datasets. This study proposes a privacy‐preserving, labeling‐free occupancy sensor using a time‐of‐flight (ToF) camera, and a clustering algorithm. Positioned above doorways, the ToF camera captures depth data that ...</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Drone, Building envelope, Envelope (radar), Systems engineering, Engineering, Architectural engineering</t>
+          <t>Cluster analysis, Bounding overwatch, Computer science, Artificial intelligence, Computer vision, occupancy detection</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4411651052</t>
+          <t>https://openalex.org/W4414092520</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>A Review of Prospects and Opportunities in Disassembly With Human–Robot Collaboration</t>
+          <t>Occupant-Detection-Based Individual Control of Four-Way Air Conditioner for Sustainable Building Energy Management</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Meng-Lun Lee; Xiao Liang; Boyi Hu; Gülcan Önel; Sara Behdad et al. (6 authors)</t>
+          <t>J H Ham; Bum‐Soo Kim; In-Woo Bae; Jaewan Joe</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Journal of Manufacturing Science and Engineering</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1115/1.4063992</t>
+          <t>https://doi.org/10.3390/su16177404</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Abstract Product disassembly plays a crucial role in the recycling, remanufacturing, and reuse of end-of-use (EoU) products. However, the current manual disassembly process is inefficient due to the complexity and variation of EoU products. While fully automating disassembly is not economically viable given the intricate nature of the task, there is potential in using human–robot collaboration (HRC) to enhance disassembly operations. HRC combines the flexibility and problem-solving abilities of ...</t>
+          <t>In this study, individual control of a four-way air conditioner was developed based on the distribution of occupants to prevent unnecessary energy consumption during room-wide control. An occupancy detection algorithm was created in Python using YOLOv5 object recognition technology to identify the occupants’ distribution in space. Recorded video data were used to test the algorithm. A simulation case study for a building energy model was conducted, assuming that this algorithm was applied using ...</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Remanufacturing, Reuse, Flexibility (engineering), Task (project management), Risk analysis (engineering), Robot</t>
+          <t>Energy consumption, Python (programming language), Thermal comfort, Air conditioning, Occupancy, occupant detection</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4388496794</t>
+          <t>https://openalex.org/W4401961351</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BIM and IFC Data Readiness for AI Integration in the Construction Industry: A Review Approach</t>
+          <t>A pilot study of occupant centric control stratum ventilation based on computer vision</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Shuzhang Du; Lei Hou; Guomin Zhang; Yongtao Tan; Peng Mao</t>
+          <t>Yihang Liu; Bin Yang; Zhang Lin</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>E3S Web of Conferences</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings14103305</t>
+          <t>https://doi.org/10.1051/e3sconf/202235601029</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Building Information Modelling (BIM) has been increasingly integrated with Artificial Intelligence (AI) solutions to automate building construction processes. However, the methods for effectively transforming data from BIM formats, such as Industry Foundation Classes (IFC), into formats suitable for AI applications still need to be explored. This paper conducts a Systematic Literature Review (SLR) following the PRISMA guidelines to analyse current data preparation approaches in BIM applications....</t>
+          <t>Indoor occupant information has an obvious influence on operating parameters of heating ventilation and air conditioning (HVAC) system, which further affects occupants’ thermal comfort and energy consumption. This pilot study proposes an occupant centric control (OCC) strategy for stratum ventilation (SV) to achieve demand control ventilation (DCV). Firstly, the computer vision sensing system and deep learning algorithm are used to detect the number of occupants in real time, and the accuracy of...</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Building information modeling, Engineering, Systems engineering, Manufacturing engineering, Engineering management, Knowledge management</t>
+          <t>HVAC, Ventilation (architecture), Thermal comfort, Cooling load, Energy consumption, occupant-centric control</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4403603993</t>
+          <t>https://openalex.org/W4293719888</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>conference-paper</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Real-Time Customer Density Analysis Using Fine-Tuned YOLOv11 for Optimized HVAC Management in Supermarkets</t>
+          <t>Modified Lightweight YOLO v8 Model for Fast and Precise Indoor Occupancy Detection</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C Santhosh; Santhiya Kalimuthu; N Adhithyaa; R Sindhu; R Yamini et al. (6 authors)</t>
+          <t>Hanyuan Zhang; Luyan Liu; Jingxue Bi; Hongbin Liu; Zetao Wen et al. (7 authors)</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>2025</v>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Applied Sciences</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/icngcs64900.2025.11183037</t>
+          <t>https://doi.org/10.3390/app16010335</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>In recent years, research on smart energy management in retail settings has grown significantly with the goal of maximizing energy use and cutting expenses. For HVAC (heating, ventilation, and air conditioning) systems, prior research has mostly concentrated on static scheduling or rule-based modifications depending on anticipated store occupancy. With this research, we provide a dynamic system that uses CCTV footage's real-time client density analysis to regulate HVAC usage in various supermark...</t>
+          <t>Fast and accurate indoor occupancy detection is critical for energy efficiency and emergency rescue in the fields of smart building and indoor positioning. However, existing image-based indoor occupancy detection models often neglect small human targets and suffer from large parameters, compromising detection accuracy, real-time performance, and deployment on resource-constrained devices. To address these issues, this study proposes a modified lightweight indoor occupancy detection model based o...</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HVAC, Computer science, Scheduling (production processes), Efficient energy use, Baseline (sea), Energy (signal processing)</t>
+          <t>Occupancy, Computer science, Software deployment, Boosting (machine learning), Real-time computing, indoor occupancy detection</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4414940680</t>
+          <t>https://openalex.org/W7117459574</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Dynamic HVAC Operations Based on Occupancy Patterns With Real-Time Vision- Based System</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Siliang Lu</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>KiltHub Repository</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1184/r1/6723290</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>An integrated heating, ventilation and air-conditioning (HVAC) system is one of the most important components to determining the energy consumption of the entire building. For commercial buildings, particularly office buildings and schools, the heating and cooling loads are largely dependent on the occupant behavioral patterns such as occupancy rates and their activities. Therefore, if HVAC systems can respond to dynamic occupancy profiles, there is a large potential to reduce energy consumption...</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Occupancy, HVAC, Computer science, Real-time computing, Computer vision, HVAC control</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W2802462092</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>An occupancy-based strategy employing computer vision for reducing cooling energy consumed in buildings</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Rania A. AlQadi; Alaa Zaghloul; Shereen A. Taie</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Bulletin of Electrical Engineering and Informatics</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.11591/eei.v10i3.3058</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>The energy expended to cool the occupied areas by air conditioners represents a substantial share of the total energy exhausted in buildings. Therefore, developing strategies to reduce this energy is crucial. One of the preponderance strategies adopted to depreciate energy consumption in buildings is the occupancy-based strategy. In this research, an innovative model was established to achieve the goal of reducing cooling energy consumed in buildings based on occupancy-based combined with a cons...</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Setpoint, Energy consumption, Energy (signal processing), Occupancy, Air conditioning, air conditioning control</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W3157345320</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Gradient Boosting-Based Residual Correction Model for Occupancy Estimation Using Channel State Information Signals in Under-Actuated Zones</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>International journal of intelligent engineering and systems</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22266/ijies2025.0831.48</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>This study proposes a robust two-stage framework for estimating occupancy in under-actuated indoor zones using WiFi Channel State Information as a non-intrusive sensing modality.These zones, marked by sparse sensor coverage and irregular airflow, present challenges for conventional detection methods.To address these, a domainspecific feature engineering pipeline is introduced, incorporating temporal, nonlinear, and spatial interaction features derived from filtered channel state information ampl...</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Residual, Computer science, Boosting (machine learning), Gradient boosting, Occupancy, occupancy estimation</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W4413066570</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>article</t>
         </is>

</xml_diff>

<commit_message>
Refresh sample output files after journal-filter test run
</commit_message>
<xml_diff>
--- a/refsfinder/papers.xlsx
+++ b/refsfinder/papers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1047,12 +1047,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Measuring Indoor Occupancy through Environmental Sensors: A Systematic Review on Sensor Deployment</t>
+          <t>Clothing Insulation Rate and Metabolic Rate Estimation for Individual Thermal Comfort Assessment in Real Life</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alma Mena-Martinez; Héctor G. Ceballos; Joanna Alvarado-Uribe</t>
+          <t>Jinsong Liu; Isak Worre Foged; Thomas Baltzer Moeslund</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1065,42 +1065,42 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s22103770</t>
+          <t>https://doi.org/10.3390/s22020619</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The COVID-19 pandemic has changed our common habits and lifestyle. Occupancy information is valued more now due to the restrictions put in place to reduce the spread of the virus. Over the years, several authors have developed methods and algorithms to detect/estimate occupancy in enclosed spaces. Similarly, different types of sensors have been installed in the places to allow this measurement. However, new researchers and practitioners often find it difficult to estimate the number of sensors t...</t>
+          <t>Satisfactory indoor thermal environments can improve working efficiencies of office staff. To build such satisfactory indoor microclimates, individual thermal comfort assessment is important, for which personal clothing insulation rate (Icl) and metabolic rate (M) need to be estimated dynamically. Therefore, this paper proposes a vision-based method. Specifically, a human tracking-by-detection framework is implemented to acquire each person’s clothing status (short-sleeved, long-sleeved), key po...</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Occupancy, Software deployment, Computer science, Wireless sensor network, Environmental monitoring, indoor occupancy detection</t>
+          <t>Metabolic rate, Clothing, Thermal comfort, Estimation, Thermal manikin, metabolic rate estimation</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4280654091</t>
+          <t>https://openalex.org/W4206317890</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Clothing Insulation Rate and Metabolic Rate Estimation for Individual Thermal Comfort Assessment in Real Life</t>
+          <t>A Survey of FPGA-Based Vision Systems for Autonomous Cars</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jinsong Liu; Isak Worre Foged; Thomas Baltzer Moeslund</t>
+          <t>David Castells‐Rufas; Vinh Ngo; Juan Borrego-Carazo; Marc Codina; Carles Sanchez et al. (7 authors)</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1108,30 +1108,30 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>IEEE Access</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s22020619</t>
+          <t>https://doi.org/10.1109/access.2022.3230282</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Satisfactory indoor thermal environments can improve working efficiencies of office staff. To build such satisfactory indoor microclimates, individual thermal comfort assessment is important, for which personal clothing insulation rate (Icl) and metabolic rate (M) need to be estimated dynamically. Therefore, this paper proposes a vision-based method. Specifically, a human tracking-by-detection framework is implemented to acquire each person’s clothing status (short-sleeved, long-sleeved), key po...</t>
+          <t>On the road to making self-driving cars a reality, academic and industrial researchers are working hard to continue to increase safety while meeting technical and regulatory constraints Understanding the surrounding environment is a fundamental task in self-driving cars. It requires combining complex computer vision algorithms. Although state-of-the-art algorithms achieve good accuracy, their implementations often require powerful computing platforms with high power consumption. In some cases, t...</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Metabolic rate, Clothing, Thermal comfort, Estimation, Thermal manikin, metabolic rate estimation</t>
+          <t>Field-programmable gate array, Computer science, Automotive industry, Implementation, Latency (audio), FPGA</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4206317890</t>
+          <t>https://openalex.org/W4312399320</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1143,12 +1143,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>A high-fidelity residential building occupancy detection dataset</t>
+          <t>Thermal Imagery Feature Extraction Techniques and the Effects on Machine Learning Models for Smart HVAC Efficiency in Building Energy</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Margarite Jacoby; Sin Yong Tan; Gregor P. Henze; Soumik Sarkar</t>
+          <t>Yaa Takyiwaa Acquaah; Balakrishna Gokaraju; Raymond Tesiero; Gregory H. Monty</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1156,78 +1156,78 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Scientific Data</t>
+          <t>Remote Sensing</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41597-021-01055-x</t>
+          <t>https://doi.org/10.3390/rs13193847</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>This paper describes development of a data acquisition system used to capture a range of occupancy related modalities from single-family residences, along with the dataset that was generated. The publicly available dataset includes: grayscale images at 32-by-32 pixels, captured every second; audio files, which have undergone processing to remove personally identifiable information; indoor environmental readings, captured every ten seconds; and ground truth binary occupancy status. The data acqui...</t>
+          <t>The control of thermostats of a heating, ventilation, and air-conditioning (HVAC) system installed in commercial and residential buildings remains a pertinent problem in building energy efficiency and thermal comfort research. The ability to determine the number of people at a particular time in an area is imperative for energy efficiency in order to condition only occupied regions and thermally deficient regions. In this study of the best features comparison for detecting the number of people i...</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Occupancy, Computer science, Ground truth, Fidelity, Modalities, human presence detection</t>
+          <t>Artificial intelligence, Computer science, Pattern recognition (psychology), Wavelet, Support vector machine, occupancy detection</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3210294652</t>
+          <t>https://openalex.org/W3204008348</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>data-paper</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>A Survey of FPGA-Based Vision Systems for Autonomous Cars</t>
+          <t>Development of CNN-based visual recognition air conditioner for smart buildings</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>David Castells‐Rufas; Vinh Ngo; Juan Borrego-Carazo; Marc Codina; Carles Sanchez et al. (7 authors)</t>
+          <t>Qian Huang; Kangli Hao</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IEEE Access</t>
+          <t>Journal of Information Technology in Construction</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/access.2022.3230282</t>
+          <t>https://doi.org/10.36680/j.itcon.2020.021</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>On the road to making self-driving cars a reality, academic and industrial researchers are working hard to continue to increase safety while meeting technical and regulatory constraints Understanding the surrounding environment is a fundamental task in self-driving cars. It requires combining complex computer vision algorithms. Although state-of-the-art algorithms achieve good accuracy, their implementations often require powerful computing platforms with high power consumption. In some cases, t...</t>
+          <t>Demand-driven heating, ventilation, and air conditioning (HVAC) operations have become very attractive in energy-efficient smart buildings. Demand-oriented HVAC control largely relies on accurate detection of building occupancy levels and locations. So far, existing building occupancy detection methods have their disadvantages, and cannot fully meet the expected performance. To address this challenge, this paper proposes a visual recognition method based on convolutional neural networks (CNN), w...</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Field-programmable gate array, Computer science, Automotive industry, Implementation, Latency (audio), FPGA</t>
+          <t>HVAC, Air conditioning, Occupancy, Building automation, Computer science, occupant detection</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4312399320</t>
+          <t>https://openalex.org/W3044090728</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1239,43 +1239,43 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Thermal Imagery Feature Extraction Techniques and the Effects on Machine Learning Models for Smart HVAC Efficiency in Building Energy</t>
+          <t>Data-Driven Ventilation and Energy Optimization in Smart Office Buildings: Insights from a High-Resolution Occupancy and Indoor Climate Dataset</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yaa Takyiwaa Acquaah; Balakrishna Gokaraju; Raymond Tesiero; Gregory H. Monty</t>
+          <t>Haidar Hosamo; Silvia Mazzetto</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Remote Sensing</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/rs13193847</t>
+          <t>https://doi.org/10.3390/su17010058</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The control of thermostats of a heating, ventilation, and air-conditioning (HVAC) system installed in commercial and residential buildings remains a pertinent problem in building energy efficiency and thermal comfort research. The ability to determine the number of people at a particular time in an area is imperative for energy efficiency in order to condition only occupied regions and thermally deficient regions. In this study of the best features comparison for detecting the number of people i...</t>
+          <t>This paper explores innovative approaches to reducing energy consumption in building ventilation systems through the implementation of adaptive control strategies. Using a publicly available high-resolution dataset spanning a full year, the study integrates real-time data on occupancy, CO2 levels, temperature, window state, and external environmental conditions. Notably, occupancy data derived from computer vision-based detection using the YOLOv5 algorithm provides an unprecedented level of gran...</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Artificial intelligence, Computer science, Pattern recognition (psychology), Wavelet, Support vector machine, occupancy detection</t>
+          <t>Occupancy, Ventilation (architecture), Architectural engineering, Environmental science, Energy (signal processing), building ventilation</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3204008348</t>
+          <t>https://openalex.org/W4405781739</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1287,43 +1287,43 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Development of CNN-based visual recognition air conditioner for smart buildings</t>
+          <t>A Practical Multi-Sensor Cooling Demand Estimation Approach Based on Visual, Indoor and Outdoor Information Sensing</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Qian Huang; Kangli Hao</t>
+          <t>Junqi Wang; Norman C. F. Tse; Tin Yan Poon; John Yau Chung Chan</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Journal of Information Technology in Construction</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://doi.org/10.36680/j.itcon.2020.021</t>
+          <t>https://doi.org/10.3390/s18113591</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Demand-driven heating, ventilation, and air conditioning (HVAC) operations have become very attractive in energy-efficient smart buildings. Demand-oriented HVAC control largely relies on accurate detection of building occupancy levels and locations. So far, existing building occupancy detection methods have their disadvantages, and cannot fully meet the expected performance. To address this challenge, this paper proposes a visual recognition method based on convolutional neural networks (CNN), w...</t>
+          <t>The operating efficiency of heating, ventilation and air conditioning (HVAC) system is critical for building energy performance. Demand-based control is an efficient HVAC operating strategy, which can provide an appropriate level of HVAC services based on the recognition of actual cooling "demand." The cooling demand primarily relies on the accurate detection of occupancy. The current researches of demand-based HVAC control tend to detect the occupant count using cameras or other sensors, which ...</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>HVAC, Air conditioning, Occupancy, Building automation, Computer science, occupant detection</t>
+          <t>Estimation, Computer science, Real-time computing, Environmental science, Remote sensing, multi-sensor fusion</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3044090728</t>
+          <t>https://openalex.org/W2898388350</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1335,91 +1335,91 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Real operational labeled data of air handling units from office, auditorium, and hospital buildings</t>
+          <t>Occupancy heat gain detection and prediction using deep learning approach for reducing building energy demand</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Seunghyeon Wang</t>
+          <t>Paige Wenbin Tien; Shuangyu Wei; John Kaiser Calautit; Jo Darkwa; Christopher J. Wood</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Scientific Data</t>
+          <t>Journal of Sustainable Development of Energy Water and Environment Systems</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41597-025-05825-9</t>
+          <t>https://doi.org/10.13044/j.sdewes.d8.0378</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>This study aims to develop comprehensive real operational datasets from three distinct building types-a large-scale office, an auditorium, and a hospital-focusing on Air Handling Units (AHUs) equipped with Constant Air Volume (CAV) systems for Automated Fault Detection and Diagnosis (AFDD). Although a consistent methodological framework was followed, data collection and preparation processes were specifically adapted to each building's unique operational characteristics. Key procedures included:...</t>
+          <t>The use of fixed or scheduled setpoints combined with varying occupancy patterns in buildings could lead to spaces being over or under-conditioned, which may lead to significant waste in energy consumption.The present study aims to develop a vision-based deep learning method for real-time occupancy activity detection and recognition.The method enables predicting and generating real-time heat gain data, which can inform building energy management systems and heating, ventilation, and air-conditio...</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Computer science, Identification (biology), Fault detection and isolation, Data collection, Key (lock), air handling units</t>
+          <t>HVAC, Occupancy, Energy consumption, Air conditioning, Deep learning, occupancy detection</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4413593661</t>
+          <t>https://openalex.org/W3099488169</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>data-paper</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Data-Driven Ventilation and Energy Optimization in Smart Office Buildings: Insights from a High-Resolution Occupancy and Indoor Climate Dataset</t>
+          <t>An Ultra-low-power Embedded AI Fire Detection and Crowd Counting System for Indoor Areas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Haidar Hosamo; Silvia Mazzetto</t>
+          <t>Alexios Papaioannou; Charalampos S. Kouzinopoulos; Dimosthenis Ioannidis; Dimitrios K. Tzovaras</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>ACM Transactions on Embedded Computing Systems</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su17010058</t>
+          <t>https://doi.org/10.1145/3582433</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>This paper explores innovative approaches to reducing energy consumption in building ventilation systems through the implementation of adaptive control strategies. Using a publicly available high-resolution dataset spanning a full year, the study integrates real-time data on occupancy, CO2 levels, temperature, window state, and external environmental conditions. Notably, occupancy data derived from computer vision-based detection using the YOLOv5 algorithm provides an unprecedented level of gran...</t>
+          <t>Fire incidents in residential and industrial areas are often the cause of human casualties and property damage. Although there are existing systems that detect fire and monitor the presence of people in indoor areas, research on their implementation in embedded platforms is limited. This article introduces an ultra-low-power embedded system for fire detection and crowd counting using efficient deep learning methods. For the prediction of fire occurrences, environmental and gas sensor along with ...</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Occupancy, Ventilation (architecture), Architectural engineering, Environmental science, Energy (signal processing), building ventilation</t>
+          <t>Computer science, Fire detection, Deep learning, Real-time computing, Inference, fire detection</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4405781739</t>
+          <t>https://openalex.org/W4320498313</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1431,43 +1431,43 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>A Practical Multi-Sensor Cooling Demand Estimation Approach Based on Visual, Indoor and Outdoor Information Sensing</t>
+          <t>A ventilation early warning system (VEWS) for diaphanous workspaces considering COVID-19 and future pandemics scenarios</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Junqi Wang; Norman C. F. Tse; Tin Yan Poon; John Yau Chung Chan</t>
+          <t>Gonçal Costa; Oriol Arroyo; Pablo Rueda; Alan Briones</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Heliyon</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s18113591</t>
+          <t>https://doi.org/10.1016/j.heliyon.2023.e14640</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>The operating efficiency of heating, ventilation and air conditioning (HVAC) system is critical for building energy performance. Demand-based control is an efficient HVAC operating strategy, which can provide an appropriate level of HVAC services based on the recognition of actual cooling "demand." The cooling demand primarily relies on the accurate detection of occupancy. The current researches of demand-based HVAC control tend to detect the occupant count using cameras or other sensors, which ...</t>
+          <t>The COVID-19 pandemic has generated new needs due to the associated health risks and, more specifically, its rapid infection rate. Prevention measures to avoid contagions in indoor spaces, especially in office and public buildings (e.g., hospitals, public administration, educational centres, etc.), have led to the need for adequate ventilation to dilute the possible concentration of the virus. This article presents our contribution to this new challenge, namely the Ventilation Early Warning Syst...</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Estimation, Computer science, Real-time computing, Environmental science, Remote sensing, multi-sensor fusion</t>
+          <t>HVAC, Workspace, Warning system, Sustainability, Architectural engineering, HVAC control</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2898388350</t>
+          <t>https://openalex.org/W4327702769</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1479,43 +1479,43 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Occupancy heat gain detection and prediction using deep learning approach for reducing building energy demand</t>
+          <t>Advanced Power Converters and Learning in Diverse Robotic Innovation: A Review</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Paige Wenbin Tien; Shuangyu Wei; John Kaiser Calautit; Jo Darkwa; Christopher J. Wood</t>
+          <t>Rupam Singh; Varaha Satya Bharath Kurukuru; Mohammed Ali Khan</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Journal of Sustainable Development of Energy Water and Environment Systems</t>
+          <t>Energies</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://doi.org/10.13044/j.sdewes.d8.0378</t>
+          <t>https://doi.org/10.3390/en16207156</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>The use of fixed or scheduled setpoints combined with varying occupancy patterns in buildings could lead to spaces being over or under-conditioned, which may lead to significant waste in energy consumption.The present study aims to develop a vision-based deep learning method for real-time occupancy activity detection and recognition.The method enables predicting and generating real-time heat gain data, which can inform building energy management systems and heating, ventilation, and air-conditio...</t>
+          <t>This paper provides a comprehensive review of the integration of advanced power management systems and learning techniques in the field of robotics. It identifies the critical roles these areas play in reshaping the capabilities of robotic systems across diverse applications. To begin, it highlights the significance of efficient power usage in modern robotics. The paper explains how advanced power converters effectively control voltage, manage current and shape waveforms, thereby optimizing ener...</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HVAC, Occupancy, Energy consumption, Air conditioning, Deep learning, occupancy detection</t>
+          <t>Artificial intelligence, Robotics, Computer science, Flexibility (engineering), Robot, power converters</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3099488169</t>
+          <t>https://openalex.org/W4387780723</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1527,43 +1527,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>An Ultra-low-power Embedded AI Fire Detection and Crowd Counting System for Indoor Areas</t>
+          <t>A Review of the Potential of Drone-Based Approaches for Integrated Building Envelope Assessment</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alexios Papaioannou; Charalampos S. Kouzinopoulos; Dimosthenis Ioannidis; Dimitrios K. Tzovaras</t>
+          <t>Shayan Mirzabeigi; Ryan Razkenari; Paul L. Crovella</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ACM Transactions on Embedded Computing Systems</t>
+          <t>Buildings</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1145/3582433</t>
+          <t>https://doi.org/10.3390/buildings15132230</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Fire incidents in residential and industrial areas are often the cause of human casualties and property damage. Although there are existing systems that detect fire and monitor the presence of people in indoor areas, research on their implementation in embedded platforms is limited. This article introduces an ultra-low-power embedded system for fire detection and crowd counting using efficient deep learning methods. For the prediction of fire occurrences, environmental and gas sensor along with ...</t>
+          <t>The urgent need for affordable and scalable building retrofit solutions has intensified due to stringent clean energy targets. Traditional building energy audits, which are essential in assessing energy performance, are often time-consuming and costly because of the extensive field analysis required. There has been a gradual shift towards the public use of drones, which present opportunities for effective remote procedures that could disrupt a variety of built environment disciplines. Drone-base...</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Computer science, Fire detection, Deep learning, Real-time computing, Inference, fire detection</t>
+          <t>Drone, Building envelope, Envelope (radar), Systems engineering, Engineering, building energy audit</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4320498313</t>
+          <t>https://openalex.org/W4411651052</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1575,43 +1575,43 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>A ventilation early warning system (VEWS) for diaphanous workspaces considering COVID-19 and future pandemics scenarios</t>
+          <t>Design and Validation of an Edge-AI Fire Safety System with SmartThings Integration for Accelerated Detection and Targeted Suppression</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gonçal Costa; Oriol Arroyo; Pablo Rueda; Alan Briones</t>
+          <t>Seung-Jun Lee; Seung-Jun Lee; Hong-Sik Yun; Yang-Bae Sim; Sang-Hoon Lee et al. (6 authors)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Heliyon</t>
+          <t>Applied Sciences</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.heliyon.2023.e14640</t>
+          <t>https://doi.org/10.3390/app15148118</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The COVID-19 pandemic has generated new needs due to the associated health risks and, more specifically, its rapid infection rate. Prevention measures to avoid contagions in indoor spaces, especially in office and public buildings (e.g., hospitals, public administration, educational centres, etc.), have led to the need for adequate ventilation to dilute the possible concentration of the virus. This article presents our contribution to this new challenge, namely the Ventilation Early Warning Syst...</t>
+          <t>This study presents the design and validation of an integrated fire safety system that leverages edge AI, hybrid sensing, and precision suppression to overcome the latency and collateral limitations of conventional smoke detection and sprinkler systems. The proposed platform features a dual-mode sensor array for early fire recognition, motorized ventilation units for rapid smoke extraction, and a 360° directional nozzle for targeted agent discharge using a residue-free clean extinguishing agent....</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>HVAC, Workspace, Warning system, Sustainability, Architectural engineering, HVAC control</t>
+          <t>Computer science, edge AI, fire safety systems, fire detection, smoke detection, probabilistic risk assessment</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4327702769</t>
+          <t>https://openalex.org/W4412530877</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1623,56 +1623,60 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ODDS: Real-Time Object Detection Using Depth Sensors on Embedded GPUs</t>
+          <t>Embedded Real-Time Clothing Classifier Using One-Stage Methods for Saving Energy in Thermostats</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Niluthpol Chowdhury Mithun; Sirajum Munir; Karen Guo; Charles Shelton</t>
+          <t>Adán Medina; Juana Isabel Méndez; Pedro Ponce; Therese E. Peffer; Arturo Molina</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2018</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>2022</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/ipsn.2018.00051</t>
+          <t>https://doi.org/10.3390/en15176117</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Detecting objects that are carried when someone enters or exits a room is very useful for a wide range of smart building applications including safety, security, and energy efficiency. While there has been a significant amount of work on object recognition using large-scale RGB image datasets, RGB cameras are too privacy invasive in many smart building applications and they work poorly in the dark. Additionally, deep object detection networks require powerful and expensive GPUs. We propose a nov...</t>
+          <t>Energy-saving is a mandatory research topic since the growing population demands additional energy yearly. Moreover, climate change requires more attention to reduce the impact of generating more CO2. As a result, some new research areas need to be explored to create innovative energy-saving alternatives in electrical devices that have high energy consumption. One research area of interest is the computer visual classification for reducing energy consumption and keeping thermal comfort in thermo...</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Computer science, Convolutional neural network, Object detection, RGB color model, Deep learning, object detection</t>
+          <t>Thermostat, Energy consumption, Computer science, Clothing, HVAC, clothing classification</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2798936443</t>
+          <t>https://openalex.org/W4293030513</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>conference-paper</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Advanced Power Converters and Learning in Diverse Robotic Innovation: A Review</t>
+          <t>Testing and Evaluation of Low-Cost Sensors for Developing Open Smart Campus Systems Based on IoT</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rupam Singh; Varaha Satya Bharath Kurukuru; Mohammed Ali Khan</t>
+          <t>Pascal Neis; Dominik Warch; Max Hoppe</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1680,30 +1684,30 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Energies</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en16207156</t>
+          <t>https://doi.org/10.3390/s23208652</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>This paper provides a comprehensive review of the integration of advanced power management systems and learning techniques in the field of robotics. It identifies the critical roles these areas play in reshaping the capabilities of robotic systems across diverse applications. To begin, it highlights the significance of efficient power usage in modern robotics. The paper explains how advanced power converters effectively control voltage, manage current and shape waveforms, thereby optimizing ener...</t>
+          <t>Urbanization has led to the need for the intelligent management of various urban challenges, from traffic to energy. In this context, smart campuses and buildings emerge as microcosms of smart cities, offering both opportunities and challenges in technology and communication integration. This study sets itself apart by prioritizing sustainable, adaptable, and reusable solutions through an open-source framework and open data protocols. We utilized the Internet of Things (IoT) and cost-effective s...</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Artificial intelligence, Robotics, Computer science, Flexibility (engineering), Robot, power converters</t>
+          <t>Smart city, Computer science, Context (archaeology), Visitor pattern, Building automation, low-cost sensors</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4387780723</t>
+          <t>https://openalex.org/W4387874460</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1715,43 +1719,43 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A Review of the Potential of Drone-Based Approaches for Integrated Building Envelope Assessment</t>
+          <t>VR digital twin of office space with computer vision-based estimation of room occupancy and power consumption</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Shayan Mirzabeigi; Ryan Razkenari; Paul L. Crovella</t>
+          <t>Abhishek Mukhopadhyay; Naveen R. Talwar; Himanshu Viswakarma; G. S. Rajshekar Reddy; Shakti Srivastava et al. (7 authors)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>Discover Analytics</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings15132230</t>
+          <t>https://doi.org/10.1007/s44257-024-00008-z</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>The urgent need for affordable and scalable building retrofit solutions has intensified due to stringent clean energy targets. Traditional building energy audits, which are essential in assessing energy performance, are often time-consuming and costly because of the extensive field analysis required. There has been a gradual shift towards the public use of drones, which present opportunities for effective remote procedures that could disrupt a variety of built environment disciplines. Drone-base...</t>
+          <t>Abstract In the past years, energy consumption has increased rapidly due to many factors, including the rise in technology adoption. This has many downfalls, from higher costs to CO $$_2$$ 2 emissions. Human activities in offices and houses represent a considerable amount of energy usage. A digital twin (DT) of an open-plan common space is created, serving the purpose of remote room occupancy monitoring and automatic detection of energy consumption. A virtual reality (VR) model is developed and ...</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Drone, Building envelope, Envelope (radar), Systems engineering, Engineering, building energy audit</t>
+          <t>Algorithm, Computer science, Artificial intelligence, Machine learning, Database, digital twin</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4411651052</t>
+          <t>https://openalex.org/W4394822553</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1763,12 +1767,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Design and Validation of an Edge-AI Fire Safety System with SmartThings Integration for Accelerated Detection and Targeted Suppression</t>
+          <t>A novel lightweight skeletal temporal model for real-time, computationally efficient recognition of occupant thermal adaptation behavior</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Seung-Jun Lee; Seung-Jun Lee; Hong-Sik Yun; Yang-Bae Sim; Sang-Hoon Lee et al. (6 authors)</t>
+          <t>Zhe Wang; Hao Sun; John Kaiser Calautit; Mingda Yang; Jianbin Chen et al. (7 authors)</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1776,30 +1780,30 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Applied Sciences</t>
+          <t>Building Simulation</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/app15148118</t>
+          <t>https://doi.org/10.1007/s12273-025-1335-6</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>This study presents the design and validation of an integrated fire safety system that leverages edge AI, hybrid sensing, and precision suppression to overcome the latency and collateral limitations of conventional smoke detection and sprinkler systems. The proposed platform features a dual-mode sensor array for early fire recognition, motorized ventilation units for rapid smoke extraction, and a 360° directional nozzle for targeted agent discharge using a residue-free clean extinguishing agent....</t>
+          <t>Abstract Optimizing building energy systems based on real-time occupant behavior and feedback can lead to improved energy efficiency and enhanced thermal comfort in buildings. Traditional thermal comfort surveys do not provide real-time insights, while conventional sensors, such as thermal sensors, are limited in their ability to capture continuous, detailed occupancy data. Meanwhile, deep learning and computer vision have emerged as promising approaches for real-time occupancy behavior detectio...</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Computer science, edge AI, fire safety systems, fire detection, smoke detection, probabilistic risk assessment</t>
+          <t>Adaptation (eye), Thermal, Computer science, Artificial intelligence, Engineering, thermal comfort</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4412530877</t>
+          <t>https://openalex.org/W4413874967</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1811,43 +1815,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Embedded Real-Time Clothing Classifier Using One-Stage Methods for Saving Energy in Thermostats</t>
+          <t>IoB Internet of Things (IoT) for Smart Built Environment (SBE): Understanding the Complexity and Contributing to Energy Efficiency; A Case Study in Mediterranean Climates</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Adán Medina; Juana Isabel Méndez; Pedro Ponce; Therese E. Peffer; Arturo Molina</t>
+          <t>Ignacio Martínez Ruiz; Enrique Cano-Suñén; Álvaro Marco; Ángel Fernández</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Energies</t>
+          <t>Applied Sciences</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en15176117</t>
+          <t>https://doi.org/10.3390/app15041724</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Energy-saving is a mandatory research topic since the growing population demands additional energy yearly. Moreover, climate change requires more attention to reduce the impact of generating more CO2. As a result, some new research areas need to be explored to create innovative energy-saving alternatives in electrical devices that have high energy consumption. One research area of interest is the computer visual classification for reducing energy consumption and keeping thermal comfort in thermo...</t>
+          <t>To meet the 2050 targets about climate change and decarbonization, accomplishing thermal comfort, Internet of Things (IoT) ecosystems are key enabling technologies to move the Built Environment (BE) towards Smart Built Environment (SBE). The first contributions of this paper conceptualise SBE from its dynamic and adaptative perspectives, considering the human habitat, and enunciate SBE as a multidimensional approach through six ways of inhabiting: defensive, projective, scientific, thermodynamic...</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Thermostat, Energy consumption, Computer science, Clothing, HVAC, clothing classification</t>
+          <t>Internet of Things, Computer science, Computer security, smart built environment, energy efficiency, public buildings</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4293030513</t>
+          <t>https://openalex.org/W4407339412</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1859,12 +1863,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Testing and Evaluation of Low-Cost Sensors for Developing Open Smart Campus Systems Based on IoT</t>
+          <t>A Cost-Effective System for Indoor Three-Dimensional Occupant Positioning and Trajectory Reconstruction</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pascal Neis; Dominik Warch; Max Hoppe</t>
+          <t>Xiaomei Zhao; Shuo Li; Zhan Zhao; Honggang Li</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1872,30 +1876,30 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Buildings</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s23208652</t>
+          <t>https://doi.org/10.3390/buildings13112832</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Urbanization has led to the need for the intelligent management of various urban challenges, from traffic to energy. In this context, smart campuses and buildings emerge as microcosms of smart cities, offering both opportunities and challenges in technology and communication integration. This study sets itself apart by prioritizing sustainable, adaptable, and reusable solutions through an open-source framework and open data protocols. We utilized the Internet of Things (IoT) and cost-effective s...</t>
+          <t>Accurate indoor occupancy information extraction plays a crucial role in building energy conservation. Vision-based methods are popularly used for occupancy information extraction because of their high accuracy. However, previous vision-based methods either only provide 2D occupancy information or require expensive equipment. In this paper, we propose a cost-effective indoor occupancy information extraction system that estimates occupant positions and trajectories in 3D using a single RGB camera...</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Smart city, Computer science, Context (archaeology), Visitor pattern, Building automation, low-cost sensors</t>
+          <t>Occupancy, Computer vision, Computer science, Tracking (education), Artificial intelligence, indoor occupancy detection</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4387874460</t>
+          <t>https://openalex.org/W4388637068</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1907,43 +1911,43 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>VR digital twin of office space with computer vision-based estimation of room occupancy and power consumption</t>
+          <t>Improved human image density detection with comparison of YOLOv8 depth level architecture and drop-out implementation</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Abhishek Mukhopadhyay; Naveen R. Talwar; Himanshu Viswakarma; G. S. Rajshekar Reddy; Shakti Srivastava et al. (7 authors)</t>
+          <t>Winda Yulita; Uri Arta Ramadhani; Zunanik Mufidah; Gde KM Atmajaya; Radhinka Bagaskara et al. (7 authors)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Discover Analytics</t>
+          <t>Journal of Soft Computing Exploration</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s44257-024-00008-z</t>
+          <t>https://doi.org/10.52465/joscex.v6i1.556</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Abstract In the past years, energy consumption has increased rapidly due to many factors, including the rise in technology adoption. This has many downfalls, from higher costs to CO $$_2$$ 2 emissions. Human activities in offices and houses represent a considerable amount of energy usage. A digital twin (DT) of an open-plan common space is created, serving the purpose of remote room occupancy monitoring and automatic detection of energy consumption. A virtual reality (VR) model is developed and ...</t>
+          <t>Energy inefficiency due to Air Conditioners (AC) running in empty rooms contribute to unnecessary energy consumption and increased CO₂ emissions. This study explores how different depth levels of the YOLOv8 architecture and dropout regularization can enhance human density detection for smarter AC control systems. By evaluating model accuracy through Mean Average Precision (mAP50-95), we provide quantitative insights into how these modifications improve detection performance. Our dataset consists...</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Algorithm, Computer science, Artificial intelligence, Machine learning, Database, digital twin</t>
+          <t>Architecture, Image (mathematics), Drop (telecommunication), Computer science, Artificial intelligence, YOLOv8</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4394822553</t>
+          <t>https://openalex.org/W4409512193</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1955,43 +1959,43 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>A novel lightweight skeletal temporal model for real-time, computationally efficient recognition of occupant thermal adaptation behavior</t>
+          <t>A Lightweight Electronic Water Pump Shell Defect Detection Method Based on Improved YOLOv5s</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Zhe Wang; Hao Sun; John Kaiser Calautit; Mingda Yang; Jianbin Chen et al. (7 authors)</t>
+          <t>Qunbiao Wu; Zhen Wang; Haifeng Fang; Junji Chen; Xinfeng Wan</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Building Simulation</t>
+          <t>Computer Systems Science and Engineering</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12273-025-1335-6</t>
+          <t>https://doi.org/10.32604/csse.2023.036239</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Abstract Optimizing building energy systems based on real-time occupant behavior and feedback can lead to improved energy efficiency and enhanced thermal comfort in buildings. Traditional thermal comfort surveys do not provide real-time insights, while conventional sensors, such as thermal sensors, are limited in their ability to capture continuous, detailed occupancy data. Meanwhile, deep learning and computer vision have emerged as promising approaches for real-time occupancy behavior detectio...</t>
+          <t>For surface defects in electronic water pump shells, the manual detection efficiency is low, prone to misdetection and leak detection, and encounters problems, such as uncertainty. To improve the speed and accuracy of surface defect detection, a lightweight detection method based on an improved YOLOv5s method is proposed to replace the traditional manual detection methods. In this method, the MobileNetV3 module replaces the backbone network of YOLOv5s, depth-separable convolution is introduced, ...</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Adaptation (eye), Thermal, Computer science, Artificial intelligence, Engineering, thermal comfort</t>
+          <t>Computer science, Artificial intelligence, Pattern recognition (psychology), surface defect detection, lightweight object detection, YOLOv5</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4413874967</t>
+          <t>https://openalex.org/W4317906189</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2003,135 +2007,139 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Enhancing Energy Efficiency in Commercial Office Buildings: A Smart IoT and Machine Vision Approach</t>
+          <t>Occupancy Measurement in Under-Actuated Zones: YOLO-based Deep Learning Approach</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sushrut Madhav Patankar; Raju Kumar Swami; Sameer Suresh Nanivadekar</t>
+          <t>Ade Syahputra; Yaddarabullah Yaddarabullah; Mohammad Faiz Azhary; Aedah Binti Abd Rahman; Amna Binti Saad</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>2024</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>International Journal of Advanced Computer Science and Applications</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/wconf61366.2024.10691999</t>
+          <t>https://doi.org/10.14569/ijacsa.2024.0150277</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Commercial office buildings often waste substantial energy due to the inefficient use of HVAC and lighting systems. This paper introduces an innovative Internet of Things (IoT) and Machine Vision-based system to combat this issue and improve energy efficiency. The system combines real-time occupancy detection using the You Only Look Once (YOLO) object detection method with CCTV footage obtained through the ESP32 cam module. Additionally, machine vision technology evaluates ambient light conditio...</t>
+          <t>The challenge of accurately detecting and identifying individuals within under-actuated zones presents a relevant research problem in occupant detection. This study aims to address the challenge of occupant detection in under-actuated zones through the utilization of the You Only Look Once version 8 (YOLO v8) object detection model. The research methodology involves a comprehensive evaluation of YOLO v8's performance across three distinct zones, where its precision, accuracy, and recall capabili...</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Efficient energy use, Internet of Things, Computer science, Machine vision, Architectural engineering, commercial office buildings</t>
+          <t>Computer science, Occupancy, Deep learning, Artificial intelligence, Real-time computing, occupant detection</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4403126293</t>
+          <t>https://openalex.org/W4392404415</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>conference-paper</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Review of modern demand control solutions and technologies for HVAC operation</t>
+          <t>Privacy‐preserving labeling‐free occupancy counting sensor based on ToF camera and clustering</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Anatolijs Borodiņecs; Jurģis Zemītis; Arturs Palcikovskis; Artūrs Ardavs; Egons Lavendelis</t>
+          <t>Jaeik Jeong; Wan–Ki Park</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>E3S Web of Conferences</t>
+          <t>ETRI Journal</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1051/e3sconf/202339602020</t>
+          <t>https://doi.org/10.4218/etrij.2025-0022</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>HVAC systems, which use traditional control strategies with fixed ventilation rates or with ventilation rate schedules, do not adjust according to the required IAQ and thermal comfort. As a result, building spaces are being over or under-ventilated. In this paper, the latest modern solutions for demand-controlled HVAC system operation are analyzed, based on the review of existing studies. Such modern technologies as human detection systems, computer vision, and neural network applications are lo...</t>
+          <t>Abstract Occupancy detection systems are crucial for optimizing energy efficiency in smart cities and buildings but often face privacy and data dependency challenges. YOLO (you only look once), a widely used real‐time detection framework, relies on identifiable image data and labeled datasets. This study proposes a privacy‐preserving, labeling‐free occupancy sensor using a time‐of‐flight (ToF) camera, and a clustering algorithm. Positioned above doorways, the ToF camera captures depth data that ...</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>HVAC, Occupancy, Computer science, Indoor air quality, Building automation, demand-controlled ventilation</t>
+          <t>Cluster analysis, Bounding overwatch, Computer science, Artificial intelligence, Computer vision, occupancy detection</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4380877501</t>
+          <t>https://openalex.org/W4414092520</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>conference-paper</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IoB Internet of Things (IoT) for Smart Built Environment (SBE): Understanding the Complexity and Contributing to Energy Efficiency; A Case Study in Mediterranean Climates</t>
+          <t>Occupant-Detection-Based Individual Control of Four-Way Air Conditioner for Sustainable Building Energy Management</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ignacio Martínez Ruiz; Enrique Cano-Suñén; Álvaro Marco; Ángel Fernández</t>
+          <t>J H Ham; Bum‐Soo Kim; In-Woo Bae; Jaewan Joe</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Applied Sciences</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/app15041724</t>
+          <t>https://doi.org/10.3390/su16177404</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>To meet the 2050 targets about climate change and decarbonization, accomplishing thermal comfort, Internet of Things (IoT) ecosystems are key enabling technologies to move the Built Environment (BE) towards Smart Built Environment (SBE). The first contributions of this paper conceptualise SBE from its dynamic and adaptative perspectives, considering the human habitat, and enunciate SBE as a multidimensional approach through six ways of inhabiting: defensive, projective, scientific, thermodynamic...</t>
+          <t>In this study, individual control of a four-way air conditioner was developed based on the distribution of occupants to prevent unnecessary energy consumption during room-wide control. An occupancy detection algorithm was created in Python using YOLOv5 object recognition technology to identify the occupants’ distribution in space. Recorded video data were used to test the algorithm. A simulation case study for a building energy model was conducted, assuming that this algorithm was applied using ...</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Internet of Things, Computer science, Computer security, smart built environment, energy efficiency, public buildings</t>
+          <t>Energy consumption, Python (programming language), Thermal comfort, Air conditioning, Occupancy, occupant detection</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4407339412</t>
+          <t>https://openalex.org/W4401961351</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2143,43 +2151,43 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>A Cost-Effective System for Indoor Three-Dimensional Occupant Positioning and Trajectory Reconstruction</t>
+          <t>Modified Lightweight YOLO v8 Model for Fast and Precise Indoor Occupancy Detection</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Xiaomei Zhao; Shuo Li; Zhan Zhao; Honggang Li</t>
+          <t>Hanyuan Zhang; Luyan Liu; Jingxue Bi; Hongbin Liu; Zetao Wen et al. (7 authors)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>Applied Sciences</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/buildings13112832</t>
+          <t>https://doi.org/10.3390/app16010335</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Accurate indoor occupancy information extraction plays a crucial role in building energy conservation. Vision-based methods are popularly used for occupancy information extraction because of their high accuracy. However, previous vision-based methods either only provide 2D occupancy information or require expensive equipment. In this paper, we propose a cost-effective indoor occupancy information extraction system that estimates occupant positions and trajectories in 3D using a single RGB camera...</t>
+          <t>Fast and accurate indoor occupancy detection is critical for energy efficiency and emergency rescue in the fields of smart building and indoor positioning. However, existing image-based indoor occupancy detection models often neglect small human targets and suffer from large parameters, compromising detection accuracy, real-time performance, and deployment on resource-constrained devices. To address these issues, this study proposes a modified lightweight indoor occupancy detection model based o...</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Occupancy, Computer vision, Computer science, Tracking (education), Artificial intelligence, indoor occupancy detection</t>
+          <t>Occupancy, Computer science, Software deployment, Boosting (machine learning), Real-time computing, indoor occupancy detection</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4388637068</t>
+          <t>https://openalex.org/W7117459574</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2191,43 +2199,43 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Improved human image density detection with comparison of YOLOv8 depth level architecture and drop-out implementation</t>
+          <t>Dynamic HVAC Operations Based on Occupancy Patterns With Real-Time Vision- Based System</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Winda Yulita; Uri Arta Ramadhani; Zunanik Mufidah; Gde KM Atmajaya; Radhinka Bagaskara et al. (7 authors)</t>
+          <t>Siliang Lu</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2025</v>
+        <v>2017</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Journal of Soft Computing Exploration</t>
+          <t>KiltHub Repository</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://doi.org/10.52465/joscex.v6i1.556</t>
+          <t>https://doi.org/10.1184/r1/6723290</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Energy inefficiency due to Air Conditioners (AC) running in empty rooms contribute to unnecessary energy consumption and increased CO₂ emissions. This study explores how different depth levels of the YOLOv8 architecture and dropout regularization can enhance human density detection for smarter AC control systems. By evaluating model accuracy through Mean Average Precision (mAP50-95), we provide quantitative insights into how these modifications improve detection performance. Our dataset consists...</t>
+          <t>An integrated heating, ventilation and air-conditioning (HVAC) system is one of the most important components to determining the energy consumption of the entire building. For commercial buildings, particularly office buildings and schools, the heating and cooling loads are largely dependent on the occupant behavioral patterns such as occupancy rates and their activities. Therefore, if HVAC systems can respond to dynamic occupancy profiles, there is a large potential to reduce energy consumption...</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Architecture, Image (mathematics), Drop (telecommunication), Computer science, Artificial intelligence, YOLOv8</t>
+          <t>Occupancy, HVAC, Computer science, Real-time computing, Computer vision, HVAC control</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4409512193</t>
+          <t>https://openalex.org/W2802462092</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2239,43 +2247,43 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>A Lightweight Electronic Water Pump Shell Defect Detection Method Based on Improved YOLOv5s</t>
+          <t>An occupancy-based strategy employing computer vision for reducing cooling energy consumed in buildings</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Qunbiao Wu; Zhen Wang; Haifeng Fang; Junji Chen; Xinfeng Wan</t>
+          <t>Rania A. AlQadi; Alaa Zaghloul; Shereen A. Taie</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Computer Systems Science and Engineering</t>
+          <t>Bulletin of Electrical Engineering and Informatics</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://doi.org/10.32604/csse.2023.036239</t>
+          <t>https://doi.org/10.11591/eei.v10i3.3058</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>For surface defects in electronic water pump shells, the manual detection efficiency is low, prone to misdetection and leak detection, and encounters problems, such as uncertainty. To improve the speed and accuracy of surface defect detection, a lightweight detection method based on an improved YOLOv5s method is proposed to replace the traditional manual detection methods. In this method, the MobileNetV3 module replaces the backbone network of YOLOv5s, depth-separable convolution is introduced, ...</t>
+          <t>The energy expended to cool the occupied areas by air conditioners represents a substantial share of the total energy exhausted in buildings. Therefore, developing strategies to reduce this energy is crucial. One of the preponderance strategies adopted to depreciate energy consumption in buildings is the occupancy-based strategy. In this research, an innovative model was established to achieve the goal of reducing cooling energy consumed in buildings based on occupancy-based combined with a cons...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Computer science, Artificial intelligence, Pattern recognition (psychology), surface defect detection, lightweight object detection, YOLOv5</t>
+          <t>Setpoint, Energy consumption, Energy (signal processing), Occupancy, Air conditioning, air conditioning control</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4317906189</t>
+          <t>https://openalex.org/W3157345320</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2287,378 +2295,42 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Occupancy Measurement in Under-Actuated Zones: YOLO-based Deep Learning Approach</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Ade Syahputra; Yaddarabullah Yaddarabullah; Mohammad Faiz Azhary; Aedah Binti Abd Rahman; Amna Binti Saad</t>
-        </is>
-      </c>
+          <t>Gradient Boosting-Based Residual Correction Model for Occupancy Estimation Using Channel State Information Signals in Under-Actuated Zones</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>International Journal of Advanced Computer Science and Applications</t>
+          <t>International journal of intelligent engineering and systems</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://doi.org/10.14569/ijacsa.2024.0150277</t>
+          <t>https://doi.org/10.22266/ijies2025.0831.48</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>The challenge of accurately detecting and identifying individuals within under-actuated zones presents a relevant research problem in occupant detection. This study aims to address the challenge of occupant detection in under-actuated zones through the utilization of the You Only Look Once version 8 (YOLO v8) object detection model. The research methodology involves a comprehensive evaluation of YOLO v8's performance across three distinct zones, where its precision, accuracy, and recall capabili...</t>
+          <t>This study proposes a robust two-stage framework for estimating occupancy in under-actuated indoor zones using WiFi Channel State Information as a non-intrusive sensing modality.These zones, marked by sparse sensor coverage and irregular airflow, present challenges for conventional detection methods.To address these, a domainspecific feature engineering pipeline is introduced, incorporating temporal, nonlinear, and spatial interaction features derived from filtered channel state information ampl...</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Computer science, Occupancy, Deep learning, Artificial intelligence, Real-time computing, occupant detection</t>
+          <t>Residual, Computer science, Boosting (machine learning), Gradient boosting, Occupancy, occupancy estimation</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4392404415</t>
+          <t>https://openalex.org/W4413066570</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Privacy‐preserving labeling‐free occupancy counting sensor based on ToF camera and clustering</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Jaeik Jeong; Wan–Ki Park</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>ETRI Journal</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.4218/etrij.2025-0022</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Abstract Occupancy detection systems are crucial for optimizing energy efficiency in smart cities and buildings but often face privacy and data dependency challenges. YOLO (you only look once), a widely used real‐time detection framework, relies on identifiable image data and labeled datasets. This study proposes a privacy‐preserving, labeling‐free occupancy sensor using a time‐of‐flight (ToF) camera, and a clustering algorithm. Positioned above doorways, the ToF camera captures depth data that ...</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Cluster analysis, Bounding overwatch, Computer science, Artificial intelligence, Computer vision, occupancy detection</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4414092520</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Occupant-Detection-Based Individual Control of Four-Way Air Conditioner for Sustainable Building Energy Management</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>J H Ham; Bum‐Soo Kim; In-Woo Bae; Jaewan Joe</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Sustainability</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3390/su16177404</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>In this study, individual control of a four-way air conditioner was developed based on the distribution of occupants to prevent unnecessary energy consumption during room-wide control. An occupancy detection algorithm was created in Python using YOLOv5 object recognition technology to identify the occupants’ distribution in space. Recorded video data were used to test the algorithm. A simulation case study for a building energy model was conducted, assuming that this algorithm was applied using ...</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Energy consumption, Python (programming language), Thermal comfort, Air conditioning, Occupancy, occupant detection</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4401961351</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>A pilot study of occupant centric control stratum ventilation based on computer vision</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Yihang Liu; Bin Yang; Zhang Lin</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>E3S Web of Conferences</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1051/e3sconf/202235601029</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Indoor occupant information has an obvious influence on operating parameters of heating ventilation and air conditioning (HVAC) system, which further affects occupants’ thermal comfort and energy consumption. This pilot study proposes an occupant centric control (OCC) strategy for stratum ventilation (SV) to achieve demand control ventilation (DCV). Firstly, the computer vision sensing system and deep learning algorithm are used to detect the number of occupants in real time, and the accuracy of...</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>HVAC, Ventilation (architecture), Thermal comfort, Cooling load, Energy consumption, occupant-centric control</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4293719888</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>conference-paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Modified Lightweight YOLO v8 Model for Fast and Precise Indoor Occupancy Detection</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Hanyuan Zhang; Luyan Liu; Jingxue Bi; Hongbin Liu; Zetao Wen et al. (7 authors)</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Applied Sciences</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3390/app16010335</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Fast and accurate indoor occupancy detection is critical for energy efficiency and emergency rescue in the fields of smart building and indoor positioning. However, existing image-based indoor occupancy detection models often neglect small human targets and suffer from large parameters, compromising detection accuracy, real-time performance, and deployment on resource-constrained devices. To address these issues, this study proposes a modified lightweight indoor occupancy detection model based o...</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Occupancy, Computer science, Software deployment, Boosting (machine learning), Real-time computing, indoor occupancy detection</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W7117459574</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Dynamic HVAC Operations Based on Occupancy Patterns With Real-Time Vision- Based System</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Siliang Lu</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>KiltHub Repository</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1184/r1/6723290</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>An integrated heating, ventilation and air-conditioning (HVAC) system is one of the most important components to determining the energy consumption of the entire building. For commercial buildings, particularly office buildings and schools, the heating and cooling loads are largely dependent on the occupant behavioral patterns such as occupancy rates and their activities. Therefore, if HVAC systems can respond to dynamic occupancy profiles, there is a large potential to reduce energy consumption...</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Occupancy, HVAC, Computer science, Real-time computing, Computer vision, HVAC control</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W2802462092</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>An occupancy-based strategy employing computer vision for reducing cooling energy consumed in buildings</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Rania A. AlQadi; Alaa Zaghloul; Shereen A. Taie</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Bulletin of Electrical Engineering and Informatics</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.11591/eei.v10i3.3058</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>The energy expended to cool the occupied areas by air conditioners represents a substantial share of the total energy exhausted in buildings. Therefore, developing strategies to reduce this energy is crucial. One of the preponderance strategies adopted to depreciate energy consumption in buildings is the occupancy-based strategy. In this research, an innovative model was established to achieve the goal of reducing cooling energy consumed in buildings based on occupancy-based combined with a cons...</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Setpoint, Energy consumption, Energy (signal processing), Occupancy, Air conditioning, air conditioning control</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W3157345320</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Gradient Boosting-Based Residual Correction Model for Occupancy Estimation Using Channel State Information Signals in Under-Actuated Zones</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>International journal of intelligent engineering and systems</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.22266/ijies2025.0831.48</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>This study proposes a robust two-stage framework for estimating occupancy in under-actuated indoor zones using WiFi Channel State Information as a non-intrusive sensing modality.These zones, marked by sparse sensor coverage and irregular airflow, present challenges for conventional detection methods.To address these, a domainspecific feature engineering pipeline is introduced, incorporating temporal, nonlinear, and spatial interaction features derived from filtered channel state information ampl...</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Residual, Computer science, Boosting (machine learning), Gradient boosting, Occupancy, occupancy estimation</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4413066570</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
         <is>
           <t>article</t>
         </is>

</xml_diff>